<commit_message>
Se agrega diccionario de Issste_Curnavaca
</commit_message>
<xml_diff>
--- a/BD_RAZAMZO/DiccionarioRAZAMZO.xlsx
+++ b/BD_RAZAMZO/DiccionarioRAZAMZO.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alanp\Desktop\Diccionarios\BD_RAZAMZO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d172cac1436627d7/Escritorio/Querys-SQL/Diccionarios_SQL-Server/BD_RAZAMZO/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C86F57A8-DC00-4331-AE3A-1375CB16F1B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{C86F57A8-DC00-4331-AE3A-1375CB16F1B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{28992186-F528-4575-976E-172D7B340A42}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21240" activeTab="1" xr2:uid="{8E2E9C6D-F322-483C-8819-A4E6DB8E596C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{8E2E9C6D-F322-483C-8819-A4E6DB8E596C}"/>
   </bookViews>
   <sheets>
     <sheet name="Tablas de RAZAMZO" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13606" uniqueCount="2123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13605" uniqueCount="2123">
   <si>
     <t>max_length</t>
   </si>
@@ -6785,10 +6785,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -6800,13 +6803,10 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -6832,9 +6832,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -6872,7 +6872,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -6978,7 +6978,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -7120,7 +7120,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -7129,7 +7129,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{514E83F7-521E-4069-9F64-B79990D5EB42}">
   <dimension ref="A2:K328"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.42578125" customWidth="1"/>
     <col min="2" max="2" width="101.7109375" style="3" customWidth="1"/>
@@ -8807,7 +8807,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A8B4663-3473-4D33-A184-8BD7C3A277AB}">
   <dimension ref="B1:I3784"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="5" width="23.5703125" style="15" customWidth="1"/>
     <col min="6" max="6" width="23.5703125" style="16" customWidth="1"/>
@@ -8815,30 +8815,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B1" s="21" t="s">
+      <c r="B1" s="28" t="s">
         <v>2122</v>
       </c>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
     </row>
     <row r="2" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B3" s="21"/>
-      <c r="C3" s="21"/>
-      <c r="D3" s="21"/>
-      <c r="E3" s="21"/>
-      <c r="F3" s="21"/>
-      <c r="G3" s="21"/>
+      <c r="B3" s="28"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
+      <c r="G3" s="28"/>
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B7" s="10" t="s">
@@ -8854,11 +8854,11 @@
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B8" s="10"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="27"/>
-      <c r="E8" s="27"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="28"/>
+      <c r="C8" s="21"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="22"/>
+      <c r="F8" s="22"/>
+      <c r="G8" s="23"/>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
@@ -8890,8 +8890,8 @@
       <c r="D10" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="E10" s="11" t="s">
-        <v>7</v>
+      <c r="E10" s="11">
+        <v>23</v>
       </c>
       <c r="F10" s="12"/>
       <c r="G10" s="12"/>
@@ -9214,11 +9214,11 @@
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B32" s="10"/>
-      <c r="C32" s="26"/>
-      <c r="D32" s="27"/>
-      <c r="E32" s="27"/>
-      <c r="F32" s="27"/>
-      <c r="G32" s="28"/>
+      <c r="C32" s="21"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="22"/>
+      <c r="G32" s="23"/>
     </row>
     <row r="33" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B33" s="2" t="s">
@@ -9372,11 +9372,11 @@
     </row>
     <row r="43" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B43" s="10"/>
-      <c r="C43" s="26"/>
-      <c r="D43" s="27"/>
-      <c r="E43" s="27"/>
-      <c r="F43" s="27"/>
-      <c r="G43" s="28"/>
+      <c r="C43" s="21"/>
+      <c r="D43" s="22"/>
+      <c r="E43" s="22"/>
+      <c r="F43" s="22"/>
+      <c r="G43" s="23"/>
     </row>
     <row r="44" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B44" s="2" t="s">
@@ -9562,11 +9562,11 @@
     </row>
     <row r="56" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B56" s="10"/>
-      <c r="C56" s="26"/>
-      <c r="D56" s="27"/>
-      <c r="E56" s="27"/>
-      <c r="F56" s="27"/>
-      <c r="G56" s="28"/>
+      <c r="C56" s="21"/>
+      <c r="D56" s="22"/>
+      <c r="E56" s="22"/>
+      <c r="F56" s="22"/>
+      <c r="G56" s="23"/>
     </row>
     <row r="57" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B57" s="2" t="s">
@@ -9768,11 +9768,11 @@
     </row>
     <row r="70" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B70" s="10"/>
-      <c r="C70" s="26"/>
-      <c r="D70" s="27"/>
-      <c r="E70" s="27"/>
-      <c r="F70" s="27"/>
-      <c r="G70" s="28"/>
+      <c r="C70" s="21"/>
+      <c r="D70" s="22"/>
+      <c r="E70" s="22"/>
+      <c r="F70" s="22"/>
+      <c r="G70" s="23"/>
     </row>
     <row r="71" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B71" s="2" t="s">
@@ -9974,11 +9974,11 @@
     </row>
     <row r="84" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B84" s="10"/>
-      <c r="C84" s="26"/>
-      <c r="D84" s="27"/>
-      <c r="E84" s="27"/>
-      <c r="F84" s="27"/>
-      <c r="G84" s="28"/>
+      <c r="C84" s="21"/>
+      <c r="D84" s="22"/>
+      <c r="E84" s="22"/>
+      <c r="F84" s="22"/>
+      <c r="G84" s="23"/>
     </row>
     <row r="85" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B85" s="2" t="s">
@@ -10078,11 +10078,11 @@
     </row>
     <row r="92" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B92" s="10"/>
-      <c r="C92" s="26"/>
-      <c r="D92" s="27"/>
-      <c r="E92" s="27"/>
-      <c r="F92" s="27"/>
-      <c r="G92" s="28"/>
+      <c r="C92" s="21"/>
+      <c r="D92" s="22"/>
+      <c r="E92" s="22"/>
+      <c r="F92" s="22"/>
+      <c r="G92" s="23"/>
     </row>
     <row r="93" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B93" s="2" t="s">
@@ -10700,11 +10700,11 @@
     </row>
     <row r="131" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B131" s="10"/>
-      <c r="C131" s="26"/>
-      <c r="D131" s="27"/>
-      <c r="E131" s="27"/>
-      <c r="F131" s="27"/>
-      <c r="G131" s="28"/>
+      <c r="C131" s="21"/>
+      <c r="D131" s="22"/>
+      <c r="E131" s="22"/>
+      <c r="F131" s="22"/>
+      <c r="G131" s="23"/>
     </row>
     <row r="132" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B132" s="2" t="s">
@@ -10810,11 +10810,11 @@
     </row>
     <row r="139" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B139" s="10"/>
-      <c r="C139" s="26"/>
-      <c r="D139" s="27"/>
-      <c r="E139" s="27"/>
-      <c r="F139" s="27"/>
-      <c r="G139" s="28"/>
+      <c r="C139" s="21"/>
+      <c r="D139" s="22"/>
+      <c r="E139" s="22"/>
+      <c r="F139" s="22"/>
+      <c r="G139" s="23"/>
     </row>
     <row r="140" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B140" s="2" t="s">
@@ -10940,11 +10940,11 @@
     </row>
     <row r="148" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B148" s="10"/>
-      <c r="C148" s="26"/>
-      <c r="D148" s="27"/>
-      <c r="E148" s="27"/>
-      <c r="F148" s="27"/>
-      <c r="G148" s="28"/>
+      <c r="C148" s="21"/>
+      <c r="D148" s="22"/>
+      <c r="E148" s="22"/>
+      <c r="F148" s="22"/>
+      <c r="G148" s="23"/>
     </row>
     <row r="149" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B149" s="2" t="s">
@@ -11028,11 +11028,11 @@
     </row>
     <row r="155" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B155" s="10"/>
-      <c r="C155" s="26"/>
-      <c r="D155" s="27"/>
-      <c r="E155" s="27"/>
-      <c r="F155" s="27"/>
-      <c r="G155" s="28"/>
+      <c r="C155" s="21"/>
+      <c r="D155" s="22"/>
+      <c r="E155" s="22"/>
+      <c r="F155" s="22"/>
+      <c r="G155" s="23"/>
     </row>
     <row r="156" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B156" s="2" t="s">
@@ -11136,11 +11136,11 @@
     </row>
     <row r="163" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B163" s="10"/>
-      <c r="C163" s="26"/>
-      <c r="D163" s="27"/>
-      <c r="E163" s="27"/>
-      <c r="F163" s="27"/>
-      <c r="G163" s="28"/>
+      <c r="C163" s="21"/>
+      <c r="D163" s="22"/>
+      <c r="E163" s="22"/>
+      <c r="F163" s="22"/>
+      <c r="G163" s="23"/>
     </row>
     <row r="164" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B164" s="2" t="s">
@@ -11320,11 +11320,11 @@
     </row>
     <row r="176" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B176" s="10"/>
-      <c r="C176" s="26"/>
-      <c r="D176" s="27"/>
-      <c r="E176" s="27"/>
-      <c r="F176" s="27"/>
-      <c r="G176" s="28"/>
+      <c r="C176" s="21"/>
+      <c r="D176" s="22"/>
+      <c r="E176" s="22"/>
+      <c r="F176" s="22"/>
+      <c r="G176" s="23"/>
     </row>
     <row r="177" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B177" s="2" t="s">
@@ -11428,11 +11428,11 @@
     </row>
     <row r="184" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B184" s="10"/>
-      <c r="C184" s="26"/>
-      <c r="D184" s="27"/>
-      <c r="E184" s="27"/>
-      <c r="F184" s="27"/>
-      <c r="G184" s="28"/>
+      <c r="C184" s="21"/>
+      <c r="D184" s="22"/>
+      <c r="E184" s="22"/>
+      <c r="F184" s="22"/>
+      <c r="G184" s="23"/>
     </row>
     <row r="185" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B185" s="2" t="s">
@@ -11522,11 +11522,11 @@
     </row>
     <row r="191" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B191" s="10"/>
-      <c r="C191" s="26"/>
-      <c r="D191" s="27"/>
-      <c r="E191" s="27"/>
-      <c r="F191" s="27"/>
-      <c r="G191" s="28"/>
+      <c r="C191" s="21"/>
+      <c r="D191" s="22"/>
+      <c r="E191" s="22"/>
+      <c r="F191" s="22"/>
+      <c r="G191" s="23"/>
     </row>
     <row r="192" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B192" s="2" t="s">
@@ -11660,11 +11660,11 @@
     </row>
     <row r="201" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B201" s="10"/>
-      <c r="C201" s="26"/>
-      <c r="D201" s="27"/>
-      <c r="E201" s="27"/>
-      <c r="F201" s="27"/>
-      <c r="G201" s="28"/>
+      <c r="C201" s="21"/>
+      <c r="D201" s="22"/>
+      <c r="E201" s="22"/>
+      <c r="F201" s="22"/>
+      <c r="G201" s="23"/>
     </row>
     <row r="202" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B202" s="2" t="s">
@@ -11910,11 +11910,11 @@
     </row>
     <row r="218" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B218" s="10"/>
-      <c r="C218" s="26"/>
-      <c r="D218" s="27"/>
-      <c r="E218" s="27"/>
-      <c r="F218" s="27"/>
-      <c r="G218" s="28"/>
+      <c r="C218" s="21"/>
+      <c r="D218" s="22"/>
+      <c r="E218" s="22"/>
+      <c r="F218" s="22"/>
+      <c r="G218" s="23"/>
     </row>
     <row r="219" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B219" s="2" t="s">
@@ -12128,11 +12128,11 @@
     </row>
     <row r="233" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B233" s="10"/>
-      <c r="C233" s="26"/>
-      <c r="D233" s="27"/>
-      <c r="E233" s="27"/>
-      <c r="F233" s="27"/>
-      <c r="G233" s="28"/>
+      <c r="C233" s="21"/>
+      <c r="D233" s="22"/>
+      <c r="E233" s="22"/>
+      <c r="F233" s="22"/>
+      <c r="G233" s="23"/>
     </row>
     <row r="234" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B234" s="2" t="s">
@@ -12370,11 +12370,11 @@
     </row>
     <row r="249" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B249" s="10"/>
-      <c r="C249" s="26"/>
-      <c r="D249" s="27"/>
-      <c r="E249" s="27"/>
-      <c r="F249" s="27"/>
-      <c r="G249" s="28"/>
+      <c r="C249" s="21"/>
+      <c r="D249" s="22"/>
+      <c r="E249" s="22"/>
+      <c r="F249" s="22"/>
+      <c r="G249" s="23"/>
     </row>
     <row r="250" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B250" s="2" t="s">
@@ -12460,11 +12460,11 @@
     </row>
     <row r="256" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B256" s="10"/>
-      <c r="C256" s="26"/>
-      <c r="D256" s="27"/>
-      <c r="E256" s="27"/>
-      <c r="F256" s="27"/>
-      <c r="G256" s="28"/>
+      <c r="C256" s="21"/>
+      <c r="D256" s="22"/>
+      <c r="E256" s="22"/>
+      <c r="F256" s="22"/>
+      <c r="G256" s="23"/>
     </row>
     <row r="257" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B257" s="2" t="s">
@@ -12582,11 +12582,11 @@
     </row>
     <row r="265" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B265" s="10"/>
-      <c r="C265" s="26"/>
-      <c r="D265" s="27"/>
-      <c r="E265" s="27"/>
-      <c r="F265" s="27"/>
-      <c r="G265" s="28"/>
+      <c r="C265" s="21"/>
+      <c r="D265" s="22"/>
+      <c r="E265" s="22"/>
+      <c r="F265" s="22"/>
+      <c r="G265" s="23"/>
     </row>
     <row r="266" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B266" s="2" t="s">
@@ -12738,11 +12738,11 @@
     </row>
     <row r="276" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B276" s="10"/>
-      <c r="C276" s="26"/>
-      <c r="D276" s="27"/>
-      <c r="E276" s="27"/>
-      <c r="F276" s="27"/>
-      <c r="G276" s="28"/>
+      <c r="C276" s="21"/>
+      <c r="D276" s="22"/>
+      <c r="E276" s="22"/>
+      <c r="F276" s="22"/>
+      <c r="G276" s="23"/>
     </row>
     <row r="277" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B277" s="2" t="s">
@@ -12858,11 +12858,11 @@
     </row>
     <row r="285" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B285" s="10"/>
-      <c r="C285" s="26"/>
-      <c r="D285" s="27"/>
-      <c r="E285" s="27"/>
-      <c r="F285" s="27"/>
-      <c r="G285" s="28"/>
+      <c r="C285" s="21"/>
+      <c r="D285" s="22"/>
+      <c r="E285" s="22"/>
+      <c r="F285" s="22"/>
+      <c r="G285" s="23"/>
     </row>
     <row r="286" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B286" s="2" t="s">
@@ -12998,11 +12998,11 @@
     </row>
     <row r="295" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B295" s="10"/>
-      <c r="C295" s="26"/>
-      <c r="D295" s="27"/>
-      <c r="E295" s="27"/>
-      <c r="F295" s="27"/>
-      <c r="G295" s="28"/>
+      <c r="C295" s="21"/>
+      <c r="D295" s="22"/>
+      <c r="E295" s="22"/>
+      <c r="F295" s="22"/>
+      <c r="G295" s="23"/>
     </row>
     <row r="296" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B296" s="2" t="s">
@@ -13102,11 +13102,11 @@
     </row>
     <row r="303" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B303" s="10"/>
-      <c r="C303" s="26"/>
-      <c r="D303" s="27"/>
-      <c r="E303" s="27"/>
-      <c r="F303" s="27"/>
-      <c r="G303" s="28"/>
+      <c r="C303" s="21"/>
+      <c r="D303" s="22"/>
+      <c r="E303" s="22"/>
+      <c r="F303" s="22"/>
+      <c r="G303" s="23"/>
     </row>
     <row r="304" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B304" s="2" t="s">
@@ -13210,11 +13210,11 @@
     </row>
     <row r="311" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B311" s="10"/>
-      <c r="C311" s="26"/>
-      <c r="D311" s="27"/>
-      <c r="E311" s="27"/>
-      <c r="F311" s="27"/>
-      <c r="G311" s="28"/>
+      <c r="C311" s="21"/>
+      <c r="D311" s="22"/>
+      <c r="E311" s="22"/>
+      <c r="F311" s="22"/>
+      <c r="G311" s="23"/>
     </row>
     <row r="312" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B312" s="2" t="s">
@@ -13336,11 +13336,11 @@
     </row>
     <row r="320" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B320" s="10"/>
-      <c r="C320" s="26"/>
-      <c r="D320" s="27"/>
-      <c r="E320" s="27"/>
-      <c r="F320" s="27"/>
-      <c r="G320" s="28"/>
+      <c r="C320" s="21"/>
+      <c r="D320" s="22"/>
+      <c r="E320" s="22"/>
+      <c r="F320" s="22"/>
+      <c r="G320" s="23"/>
     </row>
     <row r="321" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B321" s="2" t="s">
@@ -13424,11 +13424,11 @@
     </row>
     <row r="327" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B327" s="10"/>
-      <c r="C327" s="26"/>
-      <c r="D327" s="27"/>
-      <c r="E327" s="27"/>
-      <c r="F327" s="27"/>
-      <c r="G327" s="28"/>
+      <c r="C327" s="21"/>
+      <c r="D327" s="22"/>
+      <c r="E327" s="22"/>
+      <c r="F327" s="22"/>
+      <c r="G327" s="23"/>
     </row>
     <row r="328" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B328" s="2" t="s">
@@ -13896,11 +13896,11 @@
     </row>
     <row r="357" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B357" s="10"/>
-      <c r="C357" s="26"/>
-      <c r="D357" s="27"/>
-      <c r="E357" s="27"/>
-      <c r="F357" s="27"/>
-      <c r="G357" s="28"/>
+      <c r="C357" s="21"/>
+      <c r="D357" s="22"/>
+      <c r="E357" s="22"/>
+      <c r="F357" s="22"/>
+      <c r="G357" s="23"/>
     </row>
     <row r="358" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B358" s="2" t="s">
@@ -14088,11 +14088,11 @@
     </row>
     <row r="370" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B370" s="10"/>
-      <c r="C370" s="26"/>
-      <c r="D370" s="27"/>
-      <c r="E370" s="27"/>
-      <c r="F370" s="27"/>
-      <c r="G370" s="28"/>
+      <c r="C370" s="21"/>
+      <c r="D370" s="22"/>
+      <c r="E370" s="22"/>
+      <c r="F370" s="22"/>
+      <c r="G370" s="23"/>
     </row>
     <row r="371" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B371" s="2" t="s">
@@ -14216,11 +14216,11 @@
     </row>
     <row r="379" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B379" s="10"/>
-      <c r="C379" s="26"/>
-      <c r="D379" s="27"/>
-      <c r="E379" s="27"/>
-      <c r="F379" s="27"/>
-      <c r="G379" s="28"/>
+      <c r="C379" s="21"/>
+      <c r="D379" s="22"/>
+      <c r="E379" s="22"/>
+      <c r="F379" s="22"/>
+      <c r="G379" s="23"/>
     </row>
     <row r="380" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B380" s="2" t="s">
@@ -14308,11 +14308,11 @@
     </row>
     <row r="386" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B386" s="10"/>
-      <c r="C386" s="26"/>
-      <c r="D386" s="27"/>
-      <c r="E386" s="27"/>
-      <c r="F386" s="27"/>
-      <c r="G386" s="28"/>
+      <c r="C386" s="21"/>
+      <c r="D386" s="22"/>
+      <c r="E386" s="22"/>
+      <c r="F386" s="22"/>
+      <c r="G386" s="23"/>
     </row>
     <row r="387" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B387" s="2" t="s">
@@ -14576,11 +14576,11 @@
     </row>
     <row r="404" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B404" s="10"/>
-      <c r="C404" s="26"/>
-      <c r="D404" s="27"/>
-      <c r="E404" s="27"/>
-      <c r="F404" s="27"/>
-      <c r="G404" s="28"/>
+      <c r="C404" s="21"/>
+      <c r="D404" s="22"/>
+      <c r="E404" s="22"/>
+      <c r="F404" s="22"/>
+      <c r="G404" s="23"/>
     </row>
     <row r="405" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B405" s="2" t="s">
@@ -14848,11 +14848,11 @@
     </row>
     <row r="422" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B422" s="10"/>
-      <c r="C422" s="26"/>
-      <c r="D422" s="27"/>
-      <c r="E422" s="27"/>
-      <c r="F422" s="27"/>
-      <c r="G422" s="28"/>
+      <c r="C422" s="21"/>
+      <c r="D422" s="22"/>
+      <c r="E422" s="22"/>
+      <c r="F422" s="22"/>
+      <c r="G422" s="23"/>
     </row>
     <row r="423" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B423" s="2" t="s">
@@ -14922,11 +14922,11 @@
     </row>
     <row r="428" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B428" s="10"/>
-      <c r="C428" s="26"/>
-      <c r="D428" s="27"/>
-      <c r="E428" s="27"/>
-      <c r="F428" s="27"/>
-      <c r="G428" s="28"/>
+      <c r="C428" s="21"/>
+      <c r="D428" s="22"/>
+      <c r="E428" s="22"/>
+      <c r="F428" s="22"/>
+      <c r="G428" s="23"/>
     </row>
     <row r="429" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B429" s="2" t="s">
@@ -15012,11 +15012,11 @@
     </row>
     <row r="435" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B435" s="10"/>
-      <c r="C435" s="26"/>
-      <c r="D435" s="27"/>
-      <c r="E435" s="27"/>
-      <c r="F435" s="27"/>
-      <c r="G435" s="28"/>
+      <c r="C435" s="21"/>
+      <c r="D435" s="22"/>
+      <c r="E435" s="22"/>
+      <c r="F435" s="22"/>
+      <c r="G435" s="23"/>
     </row>
     <row r="436" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B436" s="2" t="s">
@@ -15156,11 +15156,11 @@
     </row>
     <row r="445" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B445" s="10"/>
-      <c r="C445" s="26"/>
-      <c r="D445" s="27"/>
-      <c r="E445" s="27"/>
-      <c r="F445" s="27"/>
-      <c r="G445" s="28"/>
+      <c r="C445" s="21"/>
+      <c r="D445" s="22"/>
+      <c r="E445" s="22"/>
+      <c r="F445" s="22"/>
+      <c r="G445" s="23"/>
     </row>
     <row r="446" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B446" s="2" t="s">
@@ -15262,11 +15262,11 @@
     </row>
     <row r="453" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B453" s="10"/>
-      <c r="C453" s="26"/>
-      <c r="D453" s="27"/>
-      <c r="E453" s="27"/>
-      <c r="F453" s="27"/>
-      <c r="G453" s="28"/>
+      <c r="C453" s="21"/>
+      <c r="D453" s="22"/>
+      <c r="E453" s="22"/>
+      <c r="F453" s="22"/>
+      <c r="G453" s="23"/>
     </row>
     <row r="454" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B454" s="2" t="s">
@@ -15350,11 +15350,11 @@
     </row>
     <row r="460" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B460" s="10"/>
-      <c r="C460" s="26"/>
-      <c r="D460" s="27"/>
-      <c r="E460" s="27"/>
-      <c r="F460" s="27"/>
-      <c r="G460" s="28"/>
+      <c r="C460" s="21"/>
+      <c r="D460" s="22"/>
+      <c r="E460" s="22"/>
+      <c r="F460" s="22"/>
+      <c r="G460" s="23"/>
     </row>
     <row r="461" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B461" s="2" t="s">
@@ -15422,11 +15422,11 @@
     </row>
     <row r="466" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B466" s="10"/>
-      <c r="C466" s="26"/>
-      <c r="D466" s="27"/>
-      <c r="E466" s="27"/>
-      <c r="F466" s="27"/>
-      <c r="G466" s="28"/>
+      <c r="C466" s="21"/>
+      <c r="D466" s="22"/>
+      <c r="E466" s="22"/>
+      <c r="F466" s="22"/>
+      <c r="G466" s="23"/>
     </row>
     <row r="467" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B467" s="2" t="s">
@@ -15542,11 +15542,11 @@
     </row>
     <row r="475" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B475" s="10"/>
-      <c r="C475" s="26"/>
-      <c r="D475" s="27"/>
-      <c r="E475" s="27"/>
-      <c r="F475" s="27"/>
-      <c r="G475" s="28"/>
+      <c r="C475" s="21"/>
+      <c r="D475" s="22"/>
+      <c r="E475" s="22"/>
+      <c r="F475" s="22"/>
+      <c r="G475" s="23"/>
     </row>
     <row r="476" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B476" s="2" t="s">
@@ -15860,11 +15860,11 @@
     </row>
     <row r="496" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B496" s="10"/>
-      <c r="C496" s="26"/>
-      <c r="D496" s="27"/>
-      <c r="E496" s="27"/>
-      <c r="F496" s="27"/>
-      <c r="G496" s="28"/>
+      <c r="C496" s="21"/>
+      <c r="D496" s="22"/>
+      <c r="E496" s="22"/>
+      <c r="F496" s="22"/>
+      <c r="G496" s="23"/>
     </row>
     <row r="497" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B497" s="2" t="s">
@@ -16002,11 +16002,11 @@
     </row>
     <row r="506" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B506" s="10"/>
-      <c r="C506" s="26"/>
-      <c r="D506" s="27"/>
-      <c r="E506" s="27"/>
-      <c r="F506" s="27"/>
-      <c r="G506" s="28"/>
+      <c r="C506" s="21"/>
+      <c r="D506" s="22"/>
+      <c r="E506" s="22"/>
+      <c r="F506" s="22"/>
+      <c r="G506" s="23"/>
     </row>
     <row r="507" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B507" s="2" t="s">
@@ -49618,13 +49618,13 @@
       <c r="B2863" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C2863" s="23" t="s">
+      <c r="C2863" s="24" t="s">
         <v>1482</v>
       </c>
-      <c r="D2863" s="24"/>
-      <c r="E2863" s="24"/>
-      <c r="F2863" s="24"/>
-      <c r="G2863" s="25"/>
+      <c r="D2863" s="25"/>
+      <c r="E2863" s="25"/>
+      <c r="F2863" s="25"/>
+      <c r="G2863" s="26"/>
     </row>
     <row r="2864" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B2864" s="10"/>
@@ -51142,7 +51142,7 @@
       <c r="F2963" s="12"/>
       <c r="G2963" s="11"/>
     </row>
-    <row r="2964" spans="2:7" ht="255" x14ac:dyDescent="0.25">
+    <row r="2964" spans="2:7" ht="216.75" x14ac:dyDescent="0.25">
       <c r="B2964" s="11" t="s">
         <v>70</v>
       </c>
@@ -51660,21 +51660,21 @@
       <c r="B3000" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3000" s="22" t="s">
+      <c r="C3000" s="27" t="s">
         <v>1557</v>
       </c>
-      <c r="D3000" s="22"/>
-      <c r="E3000" s="22"/>
-      <c r="F3000" s="22"/>
-      <c r="G3000" s="22"/>
+      <c r="D3000" s="27"/>
+      <c r="E3000" s="27"/>
+      <c r="F3000" s="27"/>
+      <c r="G3000" s="27"/>
     </row>
     <row r="3001" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3001" s="10"/>
-      <c r="C3001" s="22"/>
-      <c r="D3001" s="22"/>
-      <c r="E3001" s="22"/>
-      <c r="F3001" s="22"/>
-      <c r="G3001" s="22"/>
+      <c r="C3001" s="27"/>
+      <c r="D3001" s="27"/>
+      <c r="E3001" s="27"/>
+      <c r="F3001" s="27"/>
+      <c r="G3001" s="27"/>
     </row>
     <row r="3002" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3002" s="2" t="s">
@@ -51830,21 +51830,21 @@
       <c r="B3012" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3012" s="22" t="s">
+      <c r="C3012" s="27" t="s">
         <v>1564</v>
       </c>
-      <c r="D3012" s="22"/>
-      <c r="E3012" s="22"/>
-      <c r="F3012" s="22"/>
-      <c r="G3012" s="22"/>
+      <c r="D3012" s="27"/>
+      <c r="E3012" s="27"/>
+      <c r="F3012" s="27"/>
+      <c r="G3012" s="27"/>
     </row>
     <row r="3013" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3013" s="10"/>
-      <c r="C3013" s="22"/>
-      <c r="D3013" s="22"/>
-      <c r="E3013" s="22"/>
-      <c r="F3013" s="22"/>
-      <c r="G3013" s="22"/>
+      <c r="C3013" s="27"/>
+      <c r="D3013" s="27"/>
+      <c r="E3013" s="27"/>
+      <c r="F3013" s="27"/>
+      <c r="G3013" s="27"/>
     </row>
     <row r="3014" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3014" s="2" t="s">
@@ -51998,21 +51998,21 @@
       <c r="B3024" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3024" s="22" t="s">
+      <c r="C3024" s="27" t="s">
         <v>1564</v>
       </c>
-      <c r="D3024" s="22"/>
-      <c r="E3024" s="22"/>
-      <c r="F3024" s="22"/>
-      <c r="G3024" s="22"/>
+      <c r="D3024" s="27"/>
+      <c r="E3024" s="27"/>
+      <c r="F3024" s="27"/>
+      <c r="G3024" s="27"/>
     </row>
     <row r="3025" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3025" s="10"/>
-      <c r="C3025" s="22"/>
-      <c r="D3025" s="22"/>
-      <c r="E3025" s="22"/>
-      <c r="F3025" s="22"/>
-      <c r="G3025" s="22"/>
+      <c r="C3025" s="27"/>
+      <c r="D3025" s="27"/>
+      <c r="E3025" s="27"/>
+      <c r="F3025" s="27"/>
+      <c r="G3025" s="27"/>
     </row>
     <row r="3026" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3026" s="2" t="s">
@@ -52166,21 +52166,21 @@
       <c r="B3036" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3036" s="22" t="s">
+      <c r="C3036" s="27" t="s">
         <v>764</v>
       </c>
-      <c r="D3036" s="22"/>
-      <c r="E3036" s="22"/>
-      <c r="F3036" s="22"/>
-      <c r="G3036" s="22"/>
+      <c r="D3036" s="27"/>
+      <c r="E3036" s="27"/>
+      <c r="F3036" s="27"/>
+      <c r="G3036" s="27"/>
     </row>
     <row r="3037" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3037" s="10"/>
-      <c r="C3037" s="22"/>
-      <c r="D3037" s="22"/>
-      <c r="E3037" s="22"/>
-      <c r="F3037" s="22"/>
-      <c r="G3037" s="22"/>
+      <c r="C3037" s="27"/>
+      <c r="D3037" s="27"/>
+      <c r="E3037" s="27"/>
+      <c r="F3037" s="27"/>
+      <c r="G3037" s="27"/>
     </row>
     <row r="3038" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3038" s="2" t="s">
@@ -52222,21 +52222,21 @@
       <c r="B3041" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3041" s="22" t="s">
+      <c r="C3041" s="27" t="s">
         <v>1570</v>
       </c>
-      <c r="D3041" s="22"/>
-      <c r="E3041" s="22"/>
-      <c r="F3041" s="22"/>
-      <c r="G3041" s="22"/>
+      <c r="D3041" s="27"/>
+      <c r="E3041" s="27"/>
+      <c r="F3041" s="27"/>
+      <c r="G3041" s="27"/>
     </row>
     <row r="3042" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3042" s="10"/>
-      <c r="C3042" s="22"/>
-      <c r="D3042" s="22"/>
-      <c r="E3042" s="22"/>
-      <c r="F3042" s="22"/>
-      <c r="G3042" s="22"/>
+      <c r="C3042" s="27"/>
+      <c r="D3042" s="27"/>
+      <c r="E3042" s="27"/>
+      <c r="F3042" s="27"/>
+      <c r="G3042" s="27"/>
     </row>
     <row r="3043" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3043" s="2" t="s">
@@ -52310,21 +52310,21 @@
       <c r="B3048" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3048" s="22" t="s">
+      <c r="C3048" s="27" t="s">
         <v>1571</v>
       </c>
-      <c r="D3048" s="22"/>
-      <c r="E3048" s="22"/>
-      <c r="F3048" s="22"/>
-      <c r="G3048" s="22"/>
+      <c r="D3048" s="27"/>
+      <c r="E3048" s="27"/>
+      <c r="F3048" s="27"/>
+      <c r="G3048" s="27"/>
     </row>
     <row r="3049" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3049" s="10"/>
-      <c r="C3049" s="22"/>
-      <c r="D3049" s="22"/>
-      <c r="E3049" s="22"/>
-      <c r="F3049" s="22"/>
-      <c r="G3049" s="22"/>
+      <c r="C3049" s="27"/>
+      <c r="D3049" s="27"/>
+      <c r="E3049" s="27"/>
+      <c r="F3049" s="27"/>
+      <c r="G3049" s="27"/>
     </row>
     <row r="3050" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3050" s="2" t="s">
@@ -52398,21 +52398,21 @@
       <c r="B3055" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3055" s="22" t="s">
+      <c r="C3055" s="27" t="s">
         <v>1572</v>
       </c>
-      <c r="D3055" s="22"/>
-      <c r="E3055" s="22"/>
-      <c r="F3055" s="22"/>
-      <c r="G3055" s="22"/>
+      <c r="D3055" s="27"/>
+      <c r="E3055" s="27"/>
+      <c r="F3055" s="27"/>
+      <c r="G3055" s="27"/>
     </row>
     <row r="3056" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3056" s="10"/>
-      <c r="C3056" s="22"/>
-      <c r="D3056" s="22"/>
-      <c r="E3056" s="22"/>
-      <c r="F3056" s="22"/>
-      <c r="G3056" s="22"/>
+      <c r="C3056" s="27"/>
+      <c r="D3056" s="27"/>
+      <c r="E3056" s="27"/>
+      <c r="F3056" s="27"/>
+      <c r="G3056" s="27"/>
     </row>
     <row r="3057" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3057" s="2" t="s">
@@ -52486,21 +52486,21 @@
       <c r="B3062" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3062" s="22" t="s">
+      <c r="C3062" s="27" t="s">
         <v>1489</v>
       </c>
-      <c r="D3062" s="22"/>
-      <c r="E3062" s="22"/>
-      <c r="F3062" s="22"/>
-      <c r="G3062" s="22"/>
+      <c r="D3062" s="27"/>
+      <c r="E3062" s="27"/>
+      <c r="F3062" s="27"/>
+      <c r="G3062" s="27"/>
     </row>
     <row r="3063" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3063" s="10"/>
-      <c r="C3063" s="22"/>
-      <c r="D3063" s="22"/>
-      <c r="E3063" s="22"/>
-      <c r="F3063" s="22"/>
-      <c r="G3063" s="22"/>
+      <c r="C3063" s="27"/>
+      <c r="D3063" s="27"/>
+      <c r="E3063" s="27"/>
+      <c r="F3063" s="27"/>
+      <c r="G3063" s="27"/>
     </row>
     <row r="3064" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3064" s="2" t="s">
@@ -52646,21 +52646,21 @@
       <c r="B3073" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3073" s="22" t="s">
+      <c r="C3073" s="27" t="s">
         <v>1581</v>
       </c>
-      <c r="D3073" s="22"/>
-      <c r="E3073" s="22"/>
-      <c r="F3073" s="22"/>
-      <c r="G3073" s="22"/>
+      <c r="D3073" s="27"/>
+      <c r="E3073" s="27"/>
+      <c r="F3073" s="27"/>
+      <c r="G3073" s="27"/>
     </row>
     <row r="3074" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3074" s="10"/>
-      <c r="C3074" s="22"/>
-      <c r="D3074" s="22"/>
-      <c r="E3074" s="22"/>
-      <c r="F3074" s="22"/>
-      <c r="G3074" s="22"/>
+      <c r="C3074" s="27"/>
+      <c r="D3074" s="27"/>
+      <c r="E3074" s="27"/>
+      <c r="F3074" s="27"/>
+      <c r="G3074" s="27"/>
     </row>
     <row r="3075" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3075" s="2" t="s">
@@ -52754,21 +52754,21 @@
       <c r="B3081" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3081" s="22" t="s">
+      <c r="C3081" s="27" t="s">
         <v>1587</v>
       </c>
-      <c r="D3081" s="22"/>
-      <c r="E3081" s="22"/>
-      <c r="F3081" s="22"/>
-      <c r="G3081" s="22"/>
+      <c r="D3081" s="27"/>
+      <c r="E3081" s="27"/>
+      <c r="F3081" s="27"/>
+      <c r="G3081" s="27"/>
     </row>
     <row r="3082" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3082" s="10"/>
-      <c r="C3082" s="22"/>
-      <c r="D3082" s="22"/>
-      <c r="E3082" s="22"/>
-      <c r="F3082" s="22"/>
-      <c r="G3082" s="22"/>
+      <c r="C3082" s="27"/>
+      <c r="D3082" s="27"/>
+      <c r="E3082" s="27"/>
+      <c r="F3082" s="27"/>
+      <c r="G3082" s="27"/>
     </row>
     <row r="3083" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3083" s="2" t="s">
@@ -52892,21 +52892,21 @@
       <c r="B3091" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3091" s="22" t="s">
+      <c r="C3091" s="27" t="s">
         <v>1589</v>
       </c>
-      <c r="D3091" s="22"/>
-      <c r="E3091" s="22"/>
-      <c r="F3091" s="22"/>
-      <c r="G3091" s="22"/>
+      <c r="D3091" s="27"/>
+      <c r="E3091" s="27"/>
+      <c r="F3091" s="27"/>
+      <c r="G3091" s="27"/>
     </row>
     <row r="3092" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3092" s="10"/>
-      <c r="C3092" s="22"/>
-      <c r="D3092" s="22"/>
-      <c r="E3092" s="22"/>
-      <c r="F3092" s="22"/>
-      <c r="G3092" s="22"/>
+      <c r="C3092" s="27"/>
+      <c r="D3092" s="27"/>
+      <c r="E3092" s="27"/>
+      <c r="F3092" s="27"/>
+      <c r="G3092" s="27"/>
     </row>
     <row r="3093" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3093" s="2" t="s">
@@ -53048,21 +53048,21 @@
       <c r="B3102" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3102" s="22" t="s">
+      <c r="C3102" s="27" t="s">
         <v>1593</v>
       </c>
-      <c r="D3102" s="22"/>
-      <c r="E3102" s="22"/>
-      <c r="F3102" s="22"/>
-      <c r="G3102" s="22"/>
+      <c r="D3102" s="27"/>
+      <c r="E3102" s="27"/>
+      <c r="F3102" s="27"/>
+      <c r="G3102" s="27"/>
     </row>
     <row r="3103" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3103" s="10"/>
-      <c r="C3103" s="22"/>
-      <c r="D3103" s="22"/>
-      <c r="E3103" s="22"/>
-      <c r="F3103" s="22"/>
-      <c r="G3103" s="22"/>
+      <c r="C3103" s="27"/>
+      <c r="D3103" s="27"/>
+      <c r="E3103" s="27"/>
+      <c r="F3103" s="27"/>
+      <c r="G3103" s="27"/>
     </row>
     <row r="3104" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3104" s="2" t="s">
@@ -53272,21 +53272,21 @@
       <c r="B3117" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3117" s="22" t="s">
+      <c r="C3117" s="27" t="s">
         <v>1600</v>
       </c>
-      <c r="D3117" s="22"/>
-      <c r="E3117" s="22"/>
-      <c r="F3117" s="22"/>
-      <c r="G3117" s="22"/>
+      <c r="D3117" s="27"/>
+      <c r="E3117" s="27"/>
+      <c r="F3117" s="27"/>
+      <c r="G3117" s="27"/>
     </row>
     <row r="3118" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3118" s="10"/>
-      <c r="C3118" s="22"/>
-      <c r="D3118" s="22"/>
-      <c r="E3118" s="22"/>
-      <c r="F3118" s="22"/>
-      <c r="G3118" s="22"/>
+      <c r="C3118" s="27"/>
+      <c r="D3118" s="27"/>
+      <c r="E3118" s="27"/>
+      <c r="F3118" s="27"/>
+      <c r="G3118" s="27"/>
     </row>
     <row r="3119" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3119" s="2" t="s">
@@ -53458,21 +53458,21 @@
       <c r="B3130" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3130" s="22" t="s">
+      <c r="C3130" s="27" t="s">
         <v>1602</v>
       </c>
-      <c r="D3130" s="22"/>
-      <c r="E3130" s="22"/>
-      <c r="F3130" s="22"/>
-      <c r="G3130" s="22"/>
+      <c r="D3130" s="27"/>
+      <c r="E3130" s="27"/>
+      <c r="F3130" s="27"/>
+      <c r="G3130" s="27"/>
     </row>
     <row r="3131" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3131" s="10"/>
-      <c r="C3131" s="22"/>
-      <c r="D3131" s="22"/>
-      <c r="E3131" s="22"/>
-      <c r="F3131" s="22"/>
-      <c r="G3131" s="22"/>
+      <c r="C3131" s="27"/>
+      <c r="D3131" s="27"/>
+      <c r="E3131" s="27"/>
+      <c r="F3131" s="27"/>
+      <c r="G3131" s="27"/>
     </row>
     <row r="3132" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3132" s="2" t="s">
@@ -53630,21 +53630,21 @@
       <c r="B3142" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3142" s="22" t="s">
+      <c r="C3142" s="27" t="s">
         <v>130</v>
       </c>
-      <c r="D3142" s="22"/>
-      <c r="E3142" s="22"/>
-      <c r="F3142" s="22"/>
-      <c r="G3142" s="22"/>
+      <c r="D3142" s="27"/>
+      <c r="E3142" s="27"/>
+      <c r="F3142" s="27"/>
+      <c r="G3142" s="27"/>
     </row>
     <row r="3143" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3143" s="10"/>
-      <c r="C3143" s="22"/>
-      <c r="D3143" s="22"/>
-      <c r="E3143" s="22"/>
-      <c r="F3143" s="22"/>
-      <c r="G3143" s="22"/>
+      <c r="C3143" s="27"/>
+      <c r="D3143" s="27"/>
+      <c r="E3143" s="27"/>
+      <c r="F3143" s="27"/>
+      <c r="G3143" s="27"/>
     </row>
     <row r="3144" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3144" s="2" t="s">
@@ -53682,7 +53682,7 @@
       <c r="F3145" s="12"/>
       <c r="G3145" s="11"/>
     </row>
-    <row r="3146" spans="2:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="3146" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3146" s="11" t="s">
         <v>74</v>
       </c>
@@ -53752,7 +53752,7 @@
       </c>
       <c r="G3149" s="11"/>
     </row>
-    <row r="3150" spans="2:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="3150" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3150" s="11" t="s">
         <v>84</v>
       </c>
@@ -53854,21 +53854,21 @@
       <c r="B3157" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3157" s="22" t="s">
+      <c r="C3157" s="27" t="s">
         <v>1584</v>
       </c>
-      <c r="D3157" s="22"/>
-      <c r="E3157" s="22"/>
-      <c r="F3157" s="22"/>
-      <c r="G3157" s="22"/>
+      <c r="D3157" s="27"/>
+      <c r="E3157" s="27"/>
+      <c r="F3157" s="27"/>
+      <c r="G3157" s="27"/>
     </row>
     <row r="3158" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3158" s="10"/>
-      <c r="C3158" s="22"/>
-      <c r="D3158" s="22"/>
-      <c r="E3158" s="22"/>
-      <c r="F3158" s="22"/>
-      <c r="G3158" s="22"/>
+      <c r="C3158" s="27"/>
+      <c r="D3158" s="27"/>
+      <c r="E3158" s="27"/>
+      <c r="F3158" s="27"/>
+      <c r="G3158" s="27"/>
     </row>
     <row r="3159" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3159" s="2" t="s">
@@ -53962,21 +53962,21 @@
       <c r="B3165" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3165" s="22" t="s">
+      <c r="C3165" s="27" t="s">
         <v>1612</v>
       </c>
-      <c r="D3165" s="22"/>
-      <c r="E3165" s="22"/>
-      <c r="F3165" s="22"/>
-      <c r="G3165" s="22"/>
+      <c r="D3165" s="27"/>
+      <c r="E3165" s="27"/>
+      <c r="F3165" s="27"/>
+      <c r="G3165" s="27"/>
     </row>
     <row r="3166" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3166" s="10"/>
-      <c r="C3166" s="22"/>
-      <c r="D3166" s="22"/>
-      <c r="E3166" s="22"/>
-      <c r="F3166" s="22"/>
-      <c r="G3166" s="22"/>
+      <c r="C3166" s="27"/>
+      <c r="D3166" s="27"/>
+      <c r="E3166" s="27"/>
+      <c r="F3166" s="27"/>
+      <c r="G3166" s="27"/>
     </row>
     <row r="3167" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3167" s="2" t="s">
@@ -54034,21 +54034,21 @@
       <c r="B3171" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3171" s="22" t="s">
+      <c r="C3171" s="27" t="s">
         <v>1613</v>
       </c>
-      <c r="D3171" s="22"/>
-      <c r="E3171" s="22"/>
-      <c r="F3171" s="22"/>
-      <c r="G3171" s="22"/>
+      <c r="D3171" s="27"/>
+      <c r="E3171" s="27"/>
+      <c r="F3171" s="27"/>
+      <c r="G3171" s="27"/>
     </row>
     <row r="3172" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3172" s="10"/>
-      <c r="C3172" s="22"/>
-      <c r="D3172" s="22"/>
-      <c r="E3172" s="22"/>
-      <c r="F3172" s="22"/>
-      <c r="G3172" s="22"/>
+      <c r="C3172" s="27"/>
+      <c r="D3172" s="27"/>
+      <c r="E3172" s="27"/>
+      <c r="F3172" s="27"/>
+      <c r="G3172" s="27"/>
     </row>
     <row r="3173" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3173" s="2" t="s">
@@ -54126,21 +54126,21 @@
       <c r="B3178" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3178" s="22" t="s">
+      <c r="C3178" s="27" t="s">
         <v>157</v>
       </c>
-      <c r="D3178" s="22"/>
-      <c r="E3178" s="22"/>
-      <c r="F3178" s="22"/>
-      <c r="G3178" s="22"/>
+      <c r="D3178" s="27"/>
+      <c r="E3178" s="27"/>
+      <c r="F3178" s="27"/>
+      <c r="G3178" s="27"/>
     </row>
     <row r="3179" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3179" s="10"/>
-      <c r="C3179" s="22"/>
-      <c r="D3179" s="22"/>
-      <c r="E3179" s="22"/>
-      <c r="F3179" s="22"/>
-      <c r="G3179" s="22"/>
+      <c r="C3179" s="27"/>
+      <c r="D3179" s="27"/>
+      <c r="E3179" s="27"/>
+      <c r="F3179" s="27"/>
+      <c r="G3179" s="27"/>
     </row>
     <row r="3180" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3180" s="2" t="s">
@@ -54278,21 +54278,21 @@
       <c r="B3189" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3189" s="22" t="s">
+      <c r="C3189" s="27" t="s">
         <v>1620</v>
       </c>
-      <c r="D3189" s="22"/>
-      <c r="E3189" s="22"/>
-      <c r="F3189" s="22"/>
-      <c r="G3189" s="22"/>
+      <c r="D3189" s="27"/>
+      <c r="E3189" s="27"/>
+      <c r="F3189" s="27"/>
+      <c r="G3189" s="27"/>
     </row>
     <row r="3190" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3190" s="10"/>
-      <c r="C3190" s="22"/>
-      <c r="D3190" s="22"/>
-      <c r="E3190" s="22"/>
-      <c r="F3190" s="22"/>
-      <c r="G3190" s="22"/>
+      <c r="C3190" s="27"/>
+      <c r="D3190" s="27"/>
+      <c r="E3190" s="27"/>
+      <c r="F3190" s="27"/>
+      <c r="G3190" s="27"/>
     </row>
     <row r="3191" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3191" s="2" t="s">
@@ -54529,21 +54529,21 @@
       <c r="B3205" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3205" s="22" t="s">
+      <c r="C3205" s="27" t="s">
         <v>1629</v>
       </c>
-      <c r="D3205" s="22"/>
-      <c r="E3205" s="22"/>
-      <c r="F3205" s="22"/>
-      <c r="G3205" s="22"/>
+      <c r="D3205" s="27"/>
+      <c r="E3205" s="27"/>
+      <c r="F3205" s="27"/>
+      <c r="G3205" s="27"/>
     </row>
     <row r="3206" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3206" s="10"/>
-      <c r="C3206" s="22"/>
-      <c r="D3206" s="22"/>
-      <c r="E3206" s="22"/>
-      <c r="F3206" s="22"/>
-      <c r="G3206" s="22"/>
+      <c r="C3206" s="27"/>
+      <c r="D3206" s="27"/>
+      <c r="E3206" s="27"/>
+      <c r="F3206" s="27"/>
+      <c r="G3206" s="27"/>
     </row>
     <row r="3207" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3207" s="2" t="s">
@@ -54667,21 +54667,21 @@
       <c r="B3215" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3215" s="22" t="s">
+      <c r="C3215" s="27" t="s">
         <v>1632</v>
       </c>
-      <c r="D3215" s="22"/>
-      <c r="E3215" s="22"/>
-      <c r="F3215" s="22"/>
-      <c r="G3215" s="22"/>
+      <c r="D3215" s="27"/>
+      <c r="E3215" s="27"/>
+      <c r="F3215" s="27"/>
+      <c r="G3215" s="27"/>
     </row>
     <row r="3216" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3216" s="10"/>
-      <c r="C3216" s="22"/>
-      <c r="D3216" s="22"/>
-      <c r="E3216" s="22"/>
-      <c r="F3216" s="22"/>
-      <c r="G3216" s="22"/>
+      <c r="C3216" s="27"/>
+      <c r="D3216" s="27"/>
+      <c r="E3216" s="27"/>
+      <c r="F3216" s="27"/>
+      <c r="G3216" s="27"/>
     </row>
     <row r="3217" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3217" s="2" t="s">
@@ -54771,21 +54771,21 @@
       <c r="B3223" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3223" s="22" t="s">
+      <c r="C3223" s="27" t="s">
         <v>955</v>
       </c>
-      <c r="D3223" s="22"/>
-      <c r="E3223" s="22"/>
-      <c r="F3223" s="22"/>
-      <c r="G3223" s="22"/>
+      <c r="D3223" s="27"/>
+      <c r="E3223" s="27"/>
+      <c r="F3223" s="27"/>
+      <c r="G3223" s="27"/>
     </row>
     <row r="3224" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3224" s="10"/>
-      <c r="C3224" s="22"/>
-      <c r="D3224" s="22"/>
-      <c r="E3224" s="22"/>
-      <c r="F3224" s="22"/>
-      <c r="G3224" s="22"/>
+      <c r="C3224" s="27"/>
+      <c r="D3224" s="27"/>
+      <c r="E3224" s="27"/>
+      <c r="F3224" s="27"/>
+      <c r="G3224" s="27"/>
     </row>
     <row r="3225" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3225" s="2" t="s">
@@ -54893,21 +54893,21 @@
       <c r="B3232" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3232" s="22" t="s">
+      <c r="C3232" s="27" t="s">
         <v>1636</v>
       </c>
-      <c r="D3232" s="22"/>
-      <c r="E3232" s="22"/>
-      <c r="F3232" s="22"/>
-      <c r="G3232" s="22"/>
+      <c r="D3232" s="27"/>
+      <c r="E3232" s="27"/>
+      <c r="F3232" s="27"/>
+      <c r="G3232" s="27"/>
     </row>
     <row r="3233" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3233" s="10"/>
-      <c r="C3233" s="22"/>
-      <c r="D3233" s="22"/>
-      <c r="E3233" s="22"/>
-      <c r="F3233" s="22"/>
-      <c r="G3233" s="22"/>
+      <c r="C3233" s="27"/>
+      <c r="D3233" s="27"/>
+      <c r="E3233" s="27"/>
+      <c r="F3233" s="27"/>
+      <c r="G3233" s="27"/>
     </row>
     <row r="3234" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3234" s="2" t="s">
@@ -55017,21 +55017,21 @@
       <c r="B3241" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3241" s="22" t="s">
+      <c r="C3241" s="27" t="s">
         <v>291</v>
       </c>
-      <c r="D3241" s="22"/>
-      <c r="E3241" s="22"/>
-      <c r="F3241" s="22"/>
-      <c r="G3241" s="22"/>
+      <c r="D3241" s="27"/>
+      <c r="E3241" s="27"/>
+      <c r="F3241" s="27"/>
+      <c r="G3241" s="27"/>
     </row>
     <row r="3242" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3242" s="10"/>
-      <c r="C3242" s="22"/>
-      <c r="D3242" s="22"/>
-      <c r="E3242" s="22"/>
-      <c r="F3242" s="22"/>
-      <c r="G3242" s="22"/>
+      <c r="C3242" s="27"/>
+      <c r="D3242" s="27"/>
+      <c r="E3242" s="27"/>
+      <c r="F3242" s="27"/>
+      <c r="G3242" s="27"/>
     </row>
     <row r="3243" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3243" s="2" t="s">
@@ -55209,21 +55209,21 @@
       <c r="B3254" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3254" s="22" t="s">
+      <c r="C3254" s="27" t="s">
         <v>1645</v>
       </c>
-      <c r="D3254" s="22"/>
-      <c r="E3254" s="22"/>
-      <c r="F3254" s="22"/>
-      <c r="G3254" s="22"/>
+      <c r="D3254" s="27"/>
+      <c r="E3254" s="27"/>
+      <c r="F3254" s="27"/>
+      <c r="G3254" s="27"/>
     </row>
     <row r="3255" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3255" s="10"/>
-      <c r="C3255" s="22"/>
-      <c r="D3255" s="22"/>
-      <c r="E3255" s="22"/>
-      <c r="F3255" s="22"/>
-      <c r="G3255" s="22"/>
+      <c r="C3255" s="27"/>
+      <c r="D3255" s="27"/>
+      <c r="E3255" s="27"/>
+      <c r="F3255" s="27"/>
+      <c r="G3255" s="27"/>
     </row>
     <row r="3256" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3256" s="2" t="s">
@@ -56203,21 +56203,21 @@
       <c r="B3317" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3317" s="22" t="s">
+      <c r="C3317" s="27" t="s">
         <v>1698</v>
       </c>
-      <c r="D3317" s="22"/>
-      <c r="E3317" s="22"/>
-      <c r="F3317" s="22"/>
-      <c r="G3317" s="22"/>
+      <c r="D3317" s="27"/>
+      <c r="E3317" s="27"/>
+      <c r="F3317" s="27"/>
+      <c r="G3317" s="27"/>
     </row>
     <row r="3318" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3318" s="10"/>
-      <c r="C3318" s="22"/>
-      <c r="D3318" s="22"/>
-      <c r="E3318" s="22"/>
-      <c r="F3318" s="22"/>
-      <c r="G3318" s="22"/>
+      <c r="C3318" s="27"/>
+      <c r="D3318" s="27"/>
+      <c r="E3318" s="27"/>
+      <c r="F3318" s="27"/>
+      <c r="G3318" s="27"/>
     </row>
     <row r="3319" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3319" s="2" t="s">
@@ -56295,21 +56295,21 @@
       <c r="B3324" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3324" s="22" t="s">
+      <c r="C3324" s="27" t="s">
         <v>1701</v>
       </c>
-      <c r="D3324" s="22"/>
-      <c r="E3324" s="22"/>
-      <c r="F3324" s="22"/>
-      <c r="G3324" s="22"/>
+      <c r="D3324" s="27"/>
+      <c r="E3324" s="27"/>
+      <c r="F3324" s="27"/>
+      <c r="G3324" s="27"/>
     </row>
     <row r="3325" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3325" s="10"/>
-      <c r="C3325" s="22"/>
-      <c r="D3325" s="22"/>
-      <c r="E3325" s="22"/>
-      <c r="F3325" s="22"/>
-      <c r="G3325" s="22"/>
+      <c r="C3325" s="27"/>
+      <c r="D3325" s="27"/>
+      <c r="E3325" s="27"/>
+      <c r="F3325" s="27"/>
+      <c r="G3325" s="27"/>
     </row>
     <row r="3326" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3326" s="2" t="s">
@@ -56387,21 +56387,21 @@
       <c r="B3331" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3331" s="22" t="s">
+      <c r="C3331" s="27" t="s">
         <v>31</v>
       </c>
-      <c r="D3331" s="22"/>
-      <c r="E3331" s="22"/>
-      <c r="F3331" s="22"/>
-      <c r="G3331" s="22"/>
+      <c r="D3331" s="27"/>
+      <c r="E3331" s="27"/>
+      <c r="F3331" s="27"/>
+      <c r="G3331" s="27"/>
     </row>
     <row r="3332" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3332" s="10"/>
-      <c r="C3332" s="22"/>
-      <c r="D3332" s="22"/>
-      <c r="E3332" s="22"/>
-      <c r="F3332" s="22"/>
-      <c r="G3332" s="22"/>
+      <c r="C3332" s="27"/>
+      <c r="D3332" s="27"/>
+      <c r="E3332" s="27"/>
+      <c r="F3332" s="27"/>
+      <c r="G3332" s="27"/>
     </row>
     <row r="3333" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3333" s="2" t="s">
@@ -56809,21 +56809,21 @@
       <c r="B3358" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3358" s="22" t="s">
+      <c r="C3358" s="27" t="s">
         <v>1719</v>
       </c>
-      <c r="D3358" s="22"/>
-      <c r="E3358" s="22"/>
-      <c r="F3358" s="22"/>
-      <c r="G3358" s="22"/>
+      <c r="D3358" s="27"/>
+      <c r="E3358" s="27"/>
+      <c r="F3358" s="27"/>
+      <c r="G3358" s="27"/>
     </row>
     <row r="3359" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3359" s="10"/>
-      <c r="C3359" s="22"/>
-      <c r="D3359" s="22"/>
-      <c r="E3359" s="22"/>
-      <c r="F3359" s="22"/>
-      <c r="G3359" s="22"/>
+      <c r="C3359" s="27"/>
+      <c r="D3359" s="27"/>
+      <c r="E3359" s="27"/>
+      <c r="F3359" s="27"/>
+      <c r="G3359" s="27"/>
     </row>
     <row r="3360" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3360" s="2" t="s">
@@ -56881,7 +56881,7 @@
         <v>1723</v>
       </c>
     </row>
-    <row r="3363" spans="2:7" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="3363" spans="2:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B3363" s="11" t="s">
         <v>1724</v>
       </c>
@@ -56937,21 +56937,21 @@
       <c r="B3367" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3367" s="22" t="s">
+      <c r="C3367" s="27" t="s">
         <v>1472</v>
       </c>
-      <c r="D3367" s="22"/>
-      <c r="E3367" s="22"/>
-      <c r="F3367" s="22"/>
-      <c r="G3367" s="22"/>
+      <c r="D3367" s="27"/>
+      <c r="E3367" s="27"/>
+      <c r="F3367" s="27"/>
+      <c r="G3367" s="27"/>
     </row>
     <row r="3368" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3368" s="10"/>
-      <c r="C3368" s="22"/>
-      <c r="D3368" s="22"/>
-      <c r="E3368" s="22"/>
-      <c r="F3368" s="22"/>
-      <c r="G3368" s="22"/>
+      <c r="C3368" s="27"/>
+      <c r="D3368" s="27"/>
+      <c r="E3368" s="27"/>
+      <c r="F3368" s="27"/>
+      <c r="G3368" s="27"/>
     </row>
     <row r="3369" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3369" s="2" t="s">
@@ -57059,7 +57059,7 @@
         <v>1730</v>
       </c>
     </row>
-    <row r="3375" spans="2:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="3375" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3375" s="11" t="s">
         <v>1731</v>
       </c>
@@ -57185,21 +57185,21 @@
       <c r="B3383" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3383" s="22" t="s">
+      <c r="C3383" s="27" t="s">
         <v>1737</v>
       </c>
-      <c r="D3383" s="22"/>
-      <c r="E3383" s="22"/>
-      <c r="F3383" s="22"/>
-      <c r="G3383" s="22"/>
+      <c r="D3383" s="27"/>
+      <c r="E3383" s="27"/>
+      <c r="F3383" s="27"/>
+      <c r="G3383" s="27"/>
     </row>
     <row r="3384" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3384" s="10"/>
-      <c r="C3384" s="22"/>
-      <c r="D3384" s="22"/>
-      <c r="E3384" s="22"/>
-      <c r="F3384" s="22"/>
-      <c r="G3384" s="22"/>
+      <c r="C3384" s="27"/>
+      <c r="D3384" s="27"/>
+      <c r="E3384" s="27"/>
+      <c r="F3384" s="27"/>
+      <c r="G3384" s="27"/>
     </row>
     <row r="3385" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3385" s="2" t="s">
@@ -57341,7 +57341,7 @@
       </c>
       <c r="G3392" s="11"/>
     </row>
-    <row r="3393" spans="2:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="3393" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3393" s="11" t="s">
         <v>591</v>
       </c>
@@ -57567,7 +57567,7 @@
       </c>
       <c r="G3405" s="11"/>
     </row>
-    <row r="3406" spans="2:7" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="3406" spans="2:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B3406" s="11" t="s">
         <v>1749</v>
       </c>
@@ -57669,21 +57669,21 @@
       <c r="B3413" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3413" s="22" t="s">
+      <c r="C3413" s="27" t="s">
         <v>1751</v>
       </c>
-      <c r="D3413" s="22"/>
-      <c r="E3413" s="22"/>
-      <c r="F3413" s="22"/>
-      <c r="G3413" s="22"/>
+      <c r="D3413" s="27"/>
+      <c r="E3413" s="27"/>
+      <c r="F3413" s="27"/>
+      <c r="G3413" s="27"/>
     </row>
     <row r="3414" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3414" s="10"/>
-      <c r="C3414" s="22"/>
-      <c r="D3414" s="22"/>
-      <c r="E3414" s="22"/>
-      <c r="F3414" s="22"/>
-      <c r="G3414" s="22"/>
+      <c r="C3414" s="27"/>
+      <c r="D3414" s="27"/>
+      <c r="E3414" s="27"/>
+      <c r="F3414" s="27"/>
+      <c r="G3414" s="27"/>
     </row>
     <row r="3415" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3415" s="2" t="s">
@@ -57777,21 +57777,21 @@
       <c r="B3421" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3421" s="22" t="s">
+      <c r="C3421" s="27" t="s">
         <v>1755</v>
       </c>
-      <c r="D3421" s="22"/>
-      <c r="E3421" s="22"/>
-      <c r="F3421" s="22"/>
-      <c r="G3421" s="22"/>
+      <c r="D3421" s="27"/>
+      <c r="E3421" s="27"/>
+      <c r="F3421" s="27"/>
+      <c r="G3421" s="27"/>
     </row>
     <row r="3422" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3422" s="10"/>
-      <c r="C3422" s="22"/>
-      <c r="D3422" s="22"/>
-      <c r="E3422" s="22"/>
-      <c r="F3422" s="22"/>
-      <c r="G3422" s="22"/>
+      <c r="C3422" s="27"/>
+      <c r="D3422" s="27"/>
+      <c r="E3422" s="27"/>
+      <c r="F3422" s="27"/>
+      <c r="G3422" s="27"/>
     </row>
     <row r="3423" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3423" s="2" t="s">
@@ -57901,21 +57901,21 @@
       <c r="B3430" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3430" s="22" t="s">
+      <c r="C3430" s="27" t="s">
         <v>1758</v>
       </c>
-      <c r="D3430" s="22"/>
-      <c r="E3430" s="22"/>
-      <c r="F3430" s="22"/>
-      <c r="G3430" s="22"/>
+      <c r="D3430" s="27"/>
+      <c r="E3430" s="27"/>
+      <c r="F3430" s="27"/>
+      <c r="G3430" s="27"/>
     </row>
     <row r="3431" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3431" s="10"/>
-      <c r="C3431" s="22"/>
-      <c r="D3431" s="22"/>
-      <c r="E3431" s="22"/>
-      <c r="F3431" s="22"/>
-      <c r="G3431" s="22"/>
+      <c r="C3431" s="27"/>
+      <c r="D3431" s="27"/>
+      <c r="E3431" s="27"/>
+      <c r="F3431" s="27"/>
+      <c r="G3431" s="27"/>
     </row>
     <row r="3432" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3432" s="2" t="s">
@@ -58023,21 +58023,21 @@
       <c r="B3439" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3439" s="22" t="s">
+      <c r="C3439" s="27" t="s">
         <v>1762</v>
       </c>
-      <c r="D3439" s="22"/>
-      <c r="E3439" s="22"/>
-      <c r="F3439" s="22"/>
-      <c r="G3439" s="22"/>
+      <c r="D3439" s="27"/>
+      <c r="E3439" s="27"/>
+      <c r="F3439" s="27"/>
+      <c r="G3439" s="27"/>
     </row>
     <row r="3440" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3440" s="10"/>
-      <c r="C3440" s="22"/>
-      <c r="D3440" s="22"/>
-      <c r="E3440" s="22"/>
-      <c r="F3440" s="22"/>
-      <c r="G3440" s="22"/>
+      <c r="C3440" s="27"/>
+      <c r="D3440" s="27"/>
+      <c r="E3440" s="27"/>
+      <c r="F3440" s="27"/>
+      <c r="G3440" s="27"/>
     </row>
     <row r="3441" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3441" s="2" t="s">
@@ -58079,21 +58079,21 @@
       <c r="B3444" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3444" s="22" t="s">
+      <c r="C3444" s="27" t="s">
         <v>573</v>
       </c>
-      <c r="D3444" s="22"/>
-      <c r="E3444" s="22"/>
-      <c r="F3444" s="22"/>
-      <c r="G3444" s="22"/>
+      <c r="D3444" s="27"/>
+      <c r="E3444" s="27"/>
+      <c r="F3444" s="27"/>
+      <c r="G3444" s="27"/>
     </row>
     <row r="3445" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3445" s="10"/>
-      <c r="C3445" s="22"/>
-      <c r="D3445" s="22"/>
-      <c r="E3445" s="22"/>
-      <c r="F3445" s="22"/>
-      <c r="G3445" s="22"/>
+      <c r="C3445" s="27"/>
+      <c r="D3445" s="27"/>
+      <c r="E3445" s="27"/>
+      <c r="F3445" s="27"/>
+      <c r="G3445" s="27"/>
     </row>
     <row r="3446" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3446" s="2" t="s">
@@ -58203,7 +58203,7 @@
       </c>
       <c r="G3451" s="11"/>
     </row>
-    <row r="3452" spans="2:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="3452" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3452" s="11" t="s">
         <v>1767</v>
       </c>
@@ -58221,7 +58221,7 @@
       </c>
       <c r="G3452" s="11"/>
     </row>
-    <row r="3453" spans="2:7" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="3453" spans="2:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B3453" s="11" t="s">
         <v>674</v>
       </c>
@@ -58255,7 +58255,7 @@
       <c r="F3454" s="12"/>
       <c r="G3454" s="11"/>
     </row>
-    <row r="3455" spans="2:7" ht="51" x14ac:dyDescent="0.25">
+    <row r="3455" spans="2:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="B3455" s="11" t="s">
         <v>315</v>
       </c>
@@ -58327,7 +58327,7 @@
       </c>
       <c r="G3458" s="11"/>
     </row>
-    <row r="3459" spans="2:7" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="3459" spans="2:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B3459" s="11" t="s">
         <v>1770</v>
       </c>
@@ -58433,21 +58433,21 @@
       <c r="B3466" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3466" s="22" t="s">
+      <c r="C3466" s="27" t="s">
         <v>1775</v>
       </c>
-      <c r="D3466" s="22"/>
-      <c r="E3466" s="22"/>
-      <c r="F3466" s="22"/>
-      <c r="G3466" s="22"/>
+      <c r="D3466" s="27"/>
+      <c r="E3466" s="27"/>
+      <c r="F3466" s="27"/>
+      <c r="G3466" s="27"/>
     </row>
     <row r="3467" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3467" s="10"/>
-      <c r="C3467" s="22"/>
-      <c r="D3467" s="22"/>
-      <c r="E3467" s="22"/>
-      <c r="F3467" s="22"/>
-      <c r="G3467" s="22"/>
+      <c r="C3467" s="27"/>
+      <c r="D3467" s="27"/>
+      <c r="E3467" s="27"/>
+      <c r="F3467" s="27"/>
+      <c r="G3467" s="27"/>
     </row>
     <row r="3468" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3468" s="2" t="s">
@@ -58525,21 +58525,21 @@
       <c r="B3473" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3473" s="22" t="s">
+      <c r="C3473" s="27" t="s">
         <v>1778</v>
       </c>
-      <c r="D3473" s="22"/>
-      <c r="E3473" s="22"/>
-      <c r="F3473" s="22"/>
-      <c r="G3473" s="22"/>
+      <c r="D3473" s="27"/>
+      <c r="E3473" s="27"/>
+      <c r="F3473" s="27"/>
+      <c r="G3473" s="27"/>
     </row>
     <row r="3474" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3474" s="10"/>
-      <c r="C3474" s="22"/>
-      <c r="D3474" s="22"/>
-      <c r="E3474" s="22"/>
-      <c r="F3474" s="22"/>
-      <c r="G3474" s="22"/>
+      <c r="C3474" s="27"/>
+      <c r="D3474" s="27"/>
+      <c r="E3474" s="27"/>
+      <c r="F3474" s="27"/>
+      <c r="G3474" s="27"/>
     </row>
     <row r="3475" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3475" s="2" t="s">
@@ -58731,21 +58731,21 @@
       <c r="B3487" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3487" s="22" t="s">
+      <c r="C3487" s="27" t="s">
         <v>576</v>
       </c>
-      <c r="D3487" s="22"/>
-      <c r="E3487" s="22"/>
-      <c r="F3487" s="22"/>
-      <c r="G3487" s="22"/>
+      <c r="D3487" s="27"/>
+      <c r="E3487" s="27"/>
+      <c r="F3487" s="27"/>
+      <c r="G3487" s="27"/>
     </row>
     <row r="3488" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3488" s="10"/>
-      <c r="C3488" s="22"/>
-      <c r="D3488" s="22"/>
-      <c r="E3488" s="22"/>
-      <c r="F3488" s="22"/>
-      <c r="G3488" s="22"/>
+      <c r="C3488" s="27"/>
+      <c r="D3488" s="27"/>
+      <c r="E3488" s="27"/>
+      <c r="F3488" s="27"/>
+      <c r="G3488" s="27"/>
     </row>
     <row r="3489" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3489" s="2" t="s">
@@ -59037,21 +59037,21 @@
       <c r="B3507" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3507" s="22" t="s">
+      <c r="C3507" s="27" t="s">
         <v>1792</v>
       </c>
-      <c r="D3507" s="22"/>
-      <c r="E3507" s="22"/>
-      <c r="F3507" s="22"/>
-      <c r="G3507" s="22"/>
+      <c r="D3507" s="27"/>
+      <c r="E3507" s="27"/>
+      <c r="F3507" s="27"/>
+      <c r="G3507" s="27"/>
     </row>
     <row r="3508" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3508" s="10"/>
-      <c r="C3508" s="22"/>
-      <c r="D3508" s="22"/>
-      <c r="E3508" s="22"/>
-      <c r="F3508" s="22"/>
-      <c r="G3508" s="22"/>
+      <c r="C3508" s="27"/>
+      <c r="D3508" s="27"/>
+      <c r="E3508" s="27"/>
+      <c r="F3508" s="27"/>
+      <c r="G3508" s="27"/>
     </row>
     <row r="3509" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3509" s="2" t="s">
@@ -59107,7 +59107,7 @@
         <v>1793</v>
       </c>
     </row>
-    <row r="3512" spans="2:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="3512" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3512" s="11" t="s">
         <v>276</v>
       </c>
@@ -59199,21 +59199,21 @@
       <c r="B3518" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3518" s="22" t="s">
+      <c r="C3518" s="27" t="s">
         <v>721</v>
       </c>
-      <c r="D3518" s="22"/>
-      <c r="E3518" s="22"/>
-      <c r="F3518" s="22"/>
-      <c r="G3518" s="22"/>
+      <c r="D3518" s="27"/>
+      <c r="E3518" s="27"/>
+      <c r="F3518" s="27"/>
+      <c r="G3518" s="27"/>
     </row>
     <row r="3519" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3519" s="10"/>
-      <c r="C3519" s="22"/>
-      <c r="D3519" s="22"/>
-      <c r="E3519" s="22"/>
-      <c r="F3519" s="22"/>
-      <c r="G3519" s="22"/>
+      <c r="C3519" s="27"/>
+      <c r="D3519" s="27"/>
+      <c r="E3519" s="27"/>
+      <c r="F3519" s="27"/>
+      <c r="G3519" s="27"/>
     </row>
     <row r="3520" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3520" s="2" t="s">
@@ -59537,21 +59537,21 @@
       <c r="B3540" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3540" s="22" t="s">
+      <c r="C3540" s="27" t="s">
         <v>1808</v>
       </c>
-      <c r="D3540" s="22"/>
-      <c r="E3540" s="22"/>
-      <c r="F3540" s="22"/>
-      <c r="G3540" s="22"/>
+      <c r="D3540" s="27"/>
+      <c r="E3540" s="27"/>
+      <c r="F3540" s="27"/>
+      <c r="G3540" s="27"/>
     </row>
     <row r="3541" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3541" s="10"/>
-      <c r="C3541" s="22"/>
-      <c r="D3541" s="22"/>
-      <c r="E3541" s="22"/>
-      <c r="F3541" s="22"/>
-      <c r="G3541" s="22"/>
+      <c r="C3541" s="27"/>
+      <c r="D3541" s="27"/>
+      <c r="E3541" s="27"/>
+      <c r="F3541" s="27"/>
+      <c r="G3541" s="27"/>
     </row>
     <row r="3542" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3542" s="2" t="s">
@@ -59675,21 +59675,21 @@
       <c r="B3550" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3550" s="22" t="s">
+      <c r="C3550" s="27" t="s">
         <v>1810</v>
       </c>
-      <c r="D3550" s="22"/>
-      <c r="E3550" s="22"/>
-      <c r="F3550" s="22"/>
-      <c r="G3550" s="22"/>
+      <c r="D3550" s="27"/>
+      <c r="E3550" s="27"/>
+      <c r="F3550" s="27"/>
+      <c r="G3550" s="27"/>
     </row>
     <row r="3551" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3551" s="10"/>
-      <c r="C3551" s="22"/>
-      <c r="D3551" s="22"/>
-      <c r="E3551" s="22"/>
-      <c r="F3551" s="22"/>
-      <c r="G3551" s="22"/>
+      <c r="C3551" s="27"/>
+      <c r="D3551" s="27"/>
+      <c r="E3551" s="27"/>
+      <c r="F3551" s="27"/>
+      <c r="G3551" s="27"/>
     </row>
     <row r="3552" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3552" s="2" t="s">
@@ -59995,21 +59995,21 @@
       <c r="B3571" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3571" s="22" t="s">
+      <c r="C3571" s="27" t="s">
         <v>1826</v>
       </c>
-      <c r="D3571" s="22"/>
-      <c r="E3571" s="22"/>
-      <c r="F3571" s="22"/>
-      <c r="G3571" s="22"/>
+      <c r="D3571" s="27"/>
+      <c r="E3571" s="27"/>
+      <c r="F3571" s="27"/>
+      <c r="G3571" s="27"/>
     </row>
     <row r="3572" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3572" s="10"/>
-      <c r="C3572" s="22"/>
-      <c r="D3572" s="22"/>
-      <c r="E3572" s="22"/>
-      <c r="F3572" s="22"/>
-      <c r="G3572" s="22"/>
+      <c r="C3572" s="27"/>
+      <c r="D3572" s="27"/>
+      <c r="E3572" s="27"/>
+      <c r="F3572" s="27"/>
+      <c r="G3572" s="27"/>
     </row>
     <row r="3573" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3573" s="2" t="s">
@@ -60137,21 +60137,21 @@
       <c r="B3581" s="10" t="s">
         <v>1942</v>
       </c>
-      <c r="C3581" s="22" t="s">
+      <c r="C3581" s="27" t="s">
         <v>1833</v>
       </c>
-      <c r="D3581" s="22"/>
-      <c r="E3581" s="22"/>
-      <c r="F3581" s="22"/>
-      <c r="G3581" s="22"/>
+      <c r="D3581" s="27"/>
+      <c r="E3581" s="27"/>
+      <c r="F3581" s="27"/>
+      <c r="G3581" s="27"/>
     </row>
     <row r="3582" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3582" s="10"/>
-      <c r="C3582" s="22"/>
-      <c r="D3582" s="22"/>
-      <c r="E3582" s="22"/>
-      <c r="F3582" s="22"/>
-      <c r="G3582" s="22"/>
+      <c r="C3582" s="27"/>
+      <c r="D3582" s="27"/>
+      <c r="E3582" s="27"/>
+      <c r="F3582" s="27"/>
+      <c r="G3582" s="27"/>
     </row>
     <row r="3583" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3583" s="2" t="s">
@@ -62993,637 +62993,6 @@
     </row>
   </sheetData>
   <mergeCells count="655">
-    <mergeCell ref="C55:G55"/>
-    <mergeCell ref="C56:G56"/>
-    <mergeCell ref="C69:G69"/>
-    <mergeCell ref="C70:G70"/>
-    <mergeCell ref="C83:G83"/>
-    <mergeCell ref="C84:G84"/>
-    <mergeCell ref="C7:G7"/>
-    <mergeCell ref="C8:G8"/>
-    <mergeCell ref="C31:G31"/>
-    <mergeCell ref="C32:G32"/>
-    <mergeCell ref="C42:G42"/>
-    <mergeCell ref="C43:G43"/>
-    <mergeCell ref="C147:G147"/>
-    <mergeCell ref="C148:G148"/>
-    <mergeCell ref="C154:G154"/>
-    <mergeCell ref="C155:G155"/>
-    <mergeCell ref="C162:G162"/>
-    <mergeCell ref="C163:G163"/>
-    <mergeCell ref="C91:G91"/>
-    <mergeCell ref="C92:G92"/>
-    <mergeCell ref="C130:G130"/>
-    <mergeCell ref="C131:G131"/>
-    <mergeCell ref="C138:G138"/>
-    <mergeCell ref="C139:G139"/>
-    <mergeCell ref="C200:G200"/>
-    <mergeCell ref="C201:G201"/>
-    <mergeCell ref="C217:G217"/>
-    <mergeCell ref="C218:G218"/>
-    <mergeCell ref="C232:G232"/>
-    <mergeCell ref="C233:G233"/>
-    <mergeCell ref="C175:G175"/>
-    <mergeCell ref="C176:G176"/>
-    <mergeCell ref="C183:G183"/>
-    <mergeCell ref="C184:G184"/>
-    <mergeCell ref="C190:G190"/>
-    <mergeCell ref="C191:G191"/>
-    <mergeCell ref="C275:G275"/>
-    <mergeCell ref="C276:G276"/>
-    <mergeCell ref="C284:G284"/>
-    <mergeCell ref="C285:G285"/>
-    <mergeCell ref="C294:G294"/>
-    <mergeCell ref="C295:G295"/>
-    <mergeCell ref="C248:G248"/>
-    <mergeCell ref="C249:G249"/>
-    <mergeCell ref="C255:G255"/>
-    <mergeCell ref="C256:G256"/>
-    <mergeCell ref="C264:G264"/>
-    <mergeCell ref="C265:G265"/>
-    <mergeCell ref="C326:G326"/>
-    <mergeCell ref="C327:G327"/>
-    <mergeCell ref="C356:G356"/>
-    <mergeCell ref="C357:G357"/>
-    <mergeCell ref="C369:G369"/>
-    <mergeCell ref="C370:G370"/>
-    <mergeCell ref="C302:G302"/>
-    <mergeCell ref="C303:G303"/>
-    <mergeCell ref="C310:G310"/>
-    <mergeCell ref="C311:G311"/>
-    <mergeCell ref="C319:G319"/>
-    <mergeCell ref="C320:G320"/>
-    <mergeCell ref="C421:G421"/>
-    <mergeCell ref="C422:G422"/>
-    <mergeCell ref="C427:G427"/>
-    <mergeCell ref="C428:G428"/>
-    <mergeCell ref="C434:G434"/>
-    <mergeCell ref="C435:G435"/>
-    <mergeCell ref="C378:G378"/>
-    <mergeCell ref="C379:G379"/>
-    <mergeCell ref="C385:G385"/>
-    <mergeCell ref="C386:G386"/>
-    <mergeCell ref="C403:G403"/>
-    <mergeCell ref="C404:G404"/>
-    <mergeCell ref="C465:G465"/>
-    <mergeCell ref="C466:G466"/>
-    <mergeCell ref="C474:G474"/>
-    <mergeCell ref="C475:G475"/>
-    <mergeCell ref="C495:G495"/>
-    <mergeCell ref="C496:G496"/>
-    <mergeCell ref="C444:G444"/>
-    <mergeCell ref="C445:G445"/>
-    <mergeCell ref="C452:G452"/>
-    <mergeCell ref="C453:G453"/>
-    <mergeCell ref="C459:G459"/>
-    <mergeCell ref="C460:G460"/>
-    <mergeCell ref="C527:G527"/>
-    <mergeCell ref="C528:G528"/>
-    <mergeCell ref="C543:G543"/>
-    <mergeCell ref="C544:G544"/>
-    <mergeCell ref="C567:G567"/>
-    <mergeCell ref="C568:G568"/>
-    <mergeCell ref="C505:G505"/>
-    <mergeCell ref="C506:G506"/>
-    <mergeCell ref="C512:G512"/>
-    <mergeCell ref="C519:G519"/>
-    <mergeCell ref="C520:G520"/>
-    <mergeCell ref="C598:G598"/>
-    <mergeCell ref="C599:G599"/>
-    <mergeCell ref="C607:G607"/>
-    <mergeCell ref="C608:G608"/>
-    <mergeCell ref="C615:G615"/>
-    <mergeCell ref="C616:G616"/>
-    <mergeCell ref="C575:G575"/>
-    <mergeCell ref="C576:G576"/>
-    <mergeCell ref="C583:G583"/>
-    <mergeCell ref="C584:G584"/>
-    <mergeCell ref="C590:G590"/>
-    <mergeCell ref="C591:G591"/>
-    <mergeCell ref="C661:G661"/>
-    <mergeCell ref="C662:G662"/>
-    <mergeCell ref="C683:G683"/>
-    <mergeCell ref="C684:G684"/>
-    <mergeCell ref="C692:G692"/>
-    <mergeCell ref="C693:G693"/>
-    <mergeCell ref="C625:G625"/>
-    <mergeCell ref="C626:G626"/>
-    <mergeCell ref="C637:G637"/>
-    <mergeCell ref="C638:G638"/>
-    <mergeCell ref="C644:G644"/>
-    <mergeCell ref="C645:G645"/>
-    <mergeCell ref="C733:G733"/>
-    <mergeCell ref="C734:G734"/>
-    <mergeCell ref="C742:G742"/>
-    <mergeCell ref="C743:G743"/>
-    <mergeCell ref="C702:G702"/>
-    <mergeCell ref="C703:G703"/>
-    <mergeCell ref="C710:G710"/>
-    <mergeCell ref="C711:G711"/>
-    <mergeCell ref="C721:G721"/>
-    <mergeCell ref="C722:G722"/>
-    <mergeCell ref="C792:G792"/>
-    <mergeCell ref="C793:G793"/>
-    <mergeCell ref="C802:G802"/>
-    <mergeCell ref="C803:G803"/>
-    <mergeCell ref="C808:G808"/>
-    <mergeCell ref="C809:G809"/>
-    <mergeCell ref="C752:G752"/>
-    <mergeCell ref="C753:G753"/>
-    <mergeCell ref="C766:G766"/>
-    <mergeCell ref="C767:G767"/>
-    <mergeCell ref="C774:G774"/>
-    <mergeCell ref="C775:G775"/>
-    <mergeCell ref="C848:G848"/>
-    <mergeCell ref="C849:G849"/>
-    <mergeCell ref="C858:G858"/>
-    <mergeCell ref="C859:G859"/>
-    <mergeCell ref="C868:G868"/>
-    <mergeCell ref="C869:G869"/>
-    <mergeCell ref="C817:G817"/>
-    <mergeCell ref="C818:G818"/>
-    <mergeCell ref="C827:G827"/>
-    <mergeCell ref="C828:G828"/>
-    <mergeCell ref="C837:G837"/>
-    <mergeCell ref="C838:G838"/>
-    <mergeCell ref="C898:G898"/>
-    <mergeCell ref="C899:G899"/>
-    <mergeCell ref="C907:G907"/>
-    <mergeCell ref="C908:G908"/>
-    <mergeCell ref="C919:G919"/>
-    <mergeCell ref="C920:G920"/>
-    <mergeCell ref="C876:G876"/>
-    <mergeCell ref="C877:G877"/>
-    <mergeCell ref="C884:G884"/>
-    <mergeCell ref="C885:G885"/>
-    <mergeCell ref="C892:G892"/>
-    <mergeCell ref="C893:G893"/>
-    <mergeCell ref="C955:G955"/>
-    <mergeCell ref="C956:G956"/>
-    <mergeCell ref="C965:G965"/>
-    <mergeCell ref="C966:G966"/>
-    <mergeCell ref="C975:G975"/>
-    <mergeCell ref="C976:G976"/>
-    <mergeCell ref="C930:G930"/>
-    <mergeCell ref="C931:G931"/>
-    <mergeCell ref="C936:G936"/>
-    <mergeCell ref="C937:G937"/>
-    <mergeCell ref="C944:G944"/>
-    <mergeCell ref="C945:G945"/>
-    <mergeCell ref="C1013:G1013"/>
-    <mergeCell ref="C1014:G1014"/>
-    <mergeCell ref="C1021:G1021"/>
-    <mergeCell ref="C1022:G1022"/>
-    <mergeCell ref="C1069:G1069"/>
-    <mergeCell ref="C1070:G1070"/>
-    <mergeCell ref="C987:G987"/>
-    <mergeCell ref="C988:G988"/>
-    <mergeCell ref="C997:G997"/>
-    <mergeCell ref="C998:G998"/>
-    <mergeCell ref="C1003:G1003"/>
-    <mergeCell ref="C1004:G1004"/>
-    <mergeCell ref="C1116:G1116"/>
-    <mergeCell ref="C1117:G1117"/>
-    <mergeCell ref="C1127:G1127"/>
-    <mergeCell ref="C1128:G1128"/>
-    <mergeCell ref="C1142:G1142"/>
-    <mergeCell ref="C1143:G1143"/>
-    <mergeCell ref="C1087:G1087"/>
-    <mergeCell ref="C1088:G1088"/>
-    <mergeCell ref="C1099:G1099"/>
-    <mergeCell ref="C1100:G1100"/>
-    <mergeCell ref="C1106:G1106"/>
-    <mergeCell ref="C1107:G1107"/>
-    <mergeCell ref="C1186:G1186"/>
-    <mergeCell ref="C1187:G1187"/>
-    <mergeCell ref="C1199:G1199"/>
-    <mergeCell ref="C1200:G1200"/>
-    <mergeCell ref="C1221:G1221"/>
-    <mergeCell ref="C1222:G1222"/>
-    <mergeCell ref="C1150:G1150"/>
-    <mergeCell ref="C1151:G1151"/>
-    <mergeCell ref="C1163:G1163"/>
-    <mergeCell ref="C1164:G1164"/>
-    <mergeCell ref="C1178:G1178"/>
-    <mergeCell ref="C1179:G1179"/>
-    <mergeCell ref="C1258:G1258"/>
-    <mergeCell ref="C1259:G1259"/>
-    <mergeCell ref="C1267:G1267"/>
-    <mergeCell ref="C1268:G1268"/>
-    <mergeCell ref="C1274:G1274"/>
-    <mergeCell ref="C1275:G1275"/>
-    <mergeCell ref="C1228:G1228"/>
-    <mergeCell ref="C1229:G1229"/>
-    <mergeCell ref="C1239:G1239"/>
-    <mergeCell ref="C1240:G1240"/>
-    <mergeCell ref="C1250:G1250"/>
-    <mergeCell ref="C1251:G1251"/>
-    <mergeCell ref="C1319:G1319"/>
-    <mergeCell ref="C1320:G1320"/>
-    <mergeCell ref="C1324:G1324"/>
-    <mergeCell ref="C1325:G1325"/>
-    <mergeCell ref="C1330:G1330"/>
-    <mergeCell ref="C1331:G1331"/>
-    <mergeCell ref="C1281:G1281"/>
-    <mergeCell ref="C1282:G1282"/>
-    <mergeCell ref="C1297:G1297"/>
-    <mergeCell ref="C1298:G1298"/>
-    <mergeCell ref="C1309:G1309"/>
-    <mergeCell ref="C1310:G1310"/>
-    <mergeCell ref="C1368:G1368"/>
-    <mergeCell ref="C1369:G1369"/>
-    <mergeCell ref="C1381:G1381"/>
-    <mergeCell ref="C1382:G1382"/>
-    <mergeCell ref="C1390:G1390"/>
-    <mergeCell ref="C1391:G1391"/>
-    <mergeCell ref="C1336:G1336"/>
-    <mergeCell ref="C1337:G1337"/>
-    <mergeCell ref="C1345:G1345"/>
-    <mergeCell ref="C1346:G1346"/>
-    <mergeCell ref="C1361:G1361"/>
-    <mergeCell ref="C1362:G1362"/>
-    <mergeCell ref="C1433:G1433"/>
-    <mergeCell ref="C1434:G1434"/>
-    <mergeCell ref="C1442:G1442"/>
-    <mergeCell ref="C1443:G1443"/>
-    <mergeCell ref="C1459:G1459"/>
-    <mergeCell ref="C1460:G1460"/>
-    <mergeCell ref="C1398:G1398"/>
-    <mergeCell ref="C1399:G1399"/>
-    <mergeCell ref="C1406:G1406"/>
-    <mergeCell ref="C1407:G1407"/>
-    <mergeCell ref="C1417:G1417"/>
-    <mergeCell ref="C1418:G1418"/>
-    <mergeCell ref="C1491:G1491"/>
-    <mergeCell ref="C1492:G1492"/>
-    <mergeCell ref="C1497:G1497"/>
-    <mergeCell ref="C1498:G1498"/>
-    <mergeCell ref="C1508:G1508"/>
-    <mergeCell ref="C1509:G1509"/>
-    <mergeCell ref="C1466:G1466"/>
-    <mergeCell ref="C1467:G1467"/>
-    <mergeCell ref="C1475:G1475"/>
-    <mergeCell ref="C1476:G1476"/>
-    <mergeCell ref="C1482:G1482"/>
-    <mergeCell ref="C1483:G1483"/>
-    <mergeCell ref="C1553:G1553"/>
-    <mergeCell ref="C1554:G1554"/>
-    <mergeCell ref="C1572:G1572"/>
-    <mergeCell ref="C1573:G1573"/>
-    <mergeCell ref="C1591:G1591"/>
-    <mergeCell ref="C1592:G1592"/>
-    <mergeCell ref="C1516:G1516"/>
-    <mergeCell ref="C1517:G1517"/>
-    <mergeCell ref="C1523:G1523"/>
-    <mergeCell ref="C1524:G1524"/>
-    <mergeCell ref="C1540:G1540"/>
-    <mergeCell ref="C1541:G1541"/>
-    <mergeCell ref="C1639:G1639"/>
-    <mergeCell ref="C1640:G1640"/>
-    <mergeCell ref="C1645:G1645"/>
-    <mergeCell ref="C1646:G1646"/>
-    <mergeCell ref="C1651:G1651"/>
-    <mergeCell ref="C1652:G1652"/>
-    <mergeCell ref="C1600:G1600"/>
-    <mergeCell ref="C1601:G1601"/>
-    <mergeCell ref="C1614:G1614"/>
-    <mergeCell ref="C1615:G1615"/>
-    <mergeCell ref="C1626:G1626"/>
-    <mergeCell ref="C1627:G1627"/>
-    <mergeCell ref="C1703:G1703"/>
-    <mergeCell ref="C1704:G1704"/>
-    <mergeCell ref="C1713:G1713"/>
-    <mergeCell ref="C1714:G1714"/>
-    <mergeCell ref="C1723:G1723"/>
-    <mergeCell ref="C1724:G1724"/>
-    <mergeCell ref="C1670:G1670"/>
-    <mergeCell ref="C1671:G1671"/>
-    <mergeCell ref="C1679:G1679"/>
-    <mergeCell ref="C1680:G1680"/>
-    <mergeCell ref="C1688:G1688"/>
-    <mergeCell ref="C1689:G1689"/>
-    <mergeCell ref="C1777:G1777"/>
-    <mergeCell ref="C1778:G1778"/>
-    <mergeCell ref="C1789:G1789"/>
-    <mergeCell ref="C1790:G1790"/>
-    <mergeCell ref="C1804:G1804"/>
-    <mergeCell ref="C1805:G1805"/>
-    <mergeCell ref="C1734:G1734"/>
-    <mergeCell ref="C1735:G1735"/>
-    <mergeCell ref="C1745:G1745"/>
-    <mergeCell ref="C1746:G1746"/>
-    <mergeCell ref="C1763:G1763"/>
-    <mergeCell ref="C1764:G1764"/>
-    <mergeCell ref="C1856:G1856"/>
-    <mergeCell ref="C1857:G1857"/>
-    <mergeCell ref="C1865:G1865"/>
-    <mergeCell ref="C1866:G1866"/>
-    <mergeCell ref="C1872:G1872"/>
-    <mergeCell ref="C1873:G1873"/>
-    <mergeCell ref="C1821:G1821"/>
-    <mergeCell ref="C1822:G1822"/>
-    <mergeCell ref="C1830:G1830"/>
-    <mergeCell ref="C1831:G1831"/>
-    <mergeCell ref="C1840:G1840"/>
-    <mergeCell ref="C1918:G1918"/>
-    <mergeCell ref="C1919:G1919"/>
-    <mergeCell ref="C1924:G1924"/>
-    <mergeCell ref="C1925:G1925"/>
-    <mergeCell ref="C1942:G1942"/>
-    <mergeCell ref="C1943:G1943"/>
-    <mergeCell ref="C1883:G1883"/>
-    <mergeCell ref="C1884:G1884"/>
-    <mergeCell ref="C1893:G1893"/>
-    <mergeCell ref="C1894:G1894"/>
-    <mergeCell ref="C1912:G1912"/>
-    <mergeCell ref="C1913:G1913"/>
-    <mergeCell ref="C1993:G1993"/>
-    <mergeCell ref="C1994:G1994"/>
-    <mergeCell ref="C2001:G2001"/>
-    <mergeCell ref="C2002:G2002"/>
-    <mergeCell ref="C2023:G2023"/>
-    <mergeCell ref="C2024:G2024"/>
-    <mergeCell ref="C1952:G1952"/>
-    <mergeCell ref="C1953:G1953"/>
-    <mergeCell ref="C1964:G1964"/>
-    <mergeCell ref="C1965:G1965"/>
-    <mergeCell ref="C1984:G1984"/>
-    <mergeCell ref="C1985:G1985"/>
-    <mergeCell ref="C2091:G2091"/>
-    <mergeCell ref="C2092:G2092"/>
-    <mergeCell ref="C2103:G2103"/>
-    <mergeCell ref="C2104:G2104"/>
-    <mergeCell ref="C2114:G2114"/>
-    <mergeCell ref="C2115:G2115"/>
-    <mergeCell ref="C2031:G2031"/>
-    <mergeCell ref="C2032:G2032"/>
-    <mergeCell ref="C2041:G2041"/>
-    <mergeCell ref="C2042:G2042"/>
-    <mergeCell ref="C2079:G2079"/>
-    <mergeCell ref="C2080:G2080"/>
-    <mergeCell ref="C2173:G2173"/>
-    <mergeCell ref="C2174:G2174"/>
-    <mergeCell ref="C2179:G2179"/>
-    <mergeCell ref="C2180:G2180"/>
-    <mergeCell ref="C2186:G2186"/>
-    <mergeCell ref="C2187:G2187"/>
-    <mergeCell ref="C2123:G2123"/>
-    <mergeCell ref="C2124:G2124"/>
-    <mergeCell ref="C2131:G2131"/>
-    <mergeCell ref="C2132:G2132"/>
-    <mergeCell ref="C2138:G2138"/>
-    <mergeCell ref="C2139:G2139"/>
-    <mergeCell ref="C2228:G2228"/>
-    <mergeCell ref="C2229:G2229"/>
-    <mergeCell ref="C2242:G2242"/>
-    <mergeCell ref="C2243:G2243"/>
-    <mergeCell ref="C2250:G2250"/>
-    <mergeCell ref="C2251:G2251"/>
-    <mergeCell ref="C2194:G2194"/>
-    <mergeCell ref="C2195:G2195"/>
-    <mergeCell ref="C2210:G2210"/>
-    <mergeCell ref="C2211:G2211"/>
-    <mergeCell ref="C2218:G2218"/>
-    <mergeCell ref="C2219:G2219"/>
-    <mergeCell ref="C2289:G2289"/>
-    <mergeCell ref="C2290:G2290"/>
-    <mergeCell ref="C2337:G2337"/>
-    <mergeCell ref="C2338:G2338"/>
-    <mergeCell ref="C2351:G2351"/>
-    <mergeCell ref="C2352:G2352"/>
-    <mergeCell ref="C2257:G2257"/>
-    <mergeCell ref="C2258:G2258"/>
-    <mergeCell ref="C2274:G2274"/>
-    <mergeCell ref="C2275:G2275"/>
-    <mergeCell ref="C2281:G2281"/>
-    <mergeCell ref="C2282:G2282"/>
-    <mergeCell ref="C2383:G2383"/>
-    <mergeCell ref="C2384:G2384"/>
-    <mergeCell ref="C2391:G2391"/>
-    <mergeCell ref="C2392:G2392"/>
-    <mergeCell ref="C2399:G2399"/>
-    <mergeCell ref="C2400:G2400"/>
-    <mergeCell ref="C2358:G2358"/>
-    <mergeCell ref="C2359:G2359"/>
-    <mergeCell ref="C2366:G2366"/>
-    <mergeCell ref="C2367:G2367"/>
-    <mergeCell ref="C2377:G2377"/>
-    <mergeCell ref="C2378:G2378"/>
-    <mergeCell ref="C2433:G2433"/>
-    <mergeCell ref="C2434:G2434"/>
-    <mergeCell ref="C2440:G2440"/>
-    <mergeCell ref="C2441:G2441"/>
-    <mergeCell ref="C2454:G2454"/>
-    <mergeCell ref="C2455:G2455"/>
-    <mergeCell ref="C2409:G2409"/>
-    <mergeCell ref="C2410:G2410"/>
-    <mergeCell ref="C2417:G2417"/>
-    <mergeCell ref="C2418:G2418"/>
-    <mergeCell ref="C2425:G2425"/>
-    <mergeCell ref="C2426:G2426"/>
-    <mergeCell ref="C2492:G2492"/>
-    <mergeCell ref="C2493:G2493"/>
-    <mergeCell ref="C2506:G2506"/>
-    <mergeCell ref="C2507:G2507"/>
-    <mergeCell ref="C2519:G2519"/>
-    <mergeCell ref="C2520:G2520"/>
-    <mergeCell ref="C2462:G2462"/>
-    <mergeCell ref="C2463:G2463"/>
-    <mergeCell ref="C2469:G2469"/>
-    <mergeCell ref="C2470:G2470"/>
-    <mergeCell ref="C2482:G2482"/>
-    <mergeCell ref="C2483:G2483"/>
-    <mergeCell ref="C2559:G2559"/>
-    <mergeCell ref="C2560:G2560"/>
-    <mergeCell ref="C2569:G2569"/>
-    <mergeCell ref="C2570:G2570"/>
-    <mergeCell ref="C2584:G2584"/>
-    <mergeCell ref="C2585:G2585"/>
-    <mergeCell ref="C2530:G2530"/>
-    <mergeCell ref="C2531:G2531"/>
-    <mergeCell ref="C2539:G2539"/>
-    <mergeCell ref="C2540:G2540"/>
-    <mergeCell ref="C2547:G2547"/>
-    <mergeCell ref="C2548:G2548"/>
-    <mergeCell ref="C2637:G2637"/>
-    <mergeCell ref="C2638:G2638"/>
-    <mergeCell ref="C2645:G2645"/>
-    <mergeCell ref="C2646:G2646"/>
-    <mergeCell ref="C2653:G2653"/>
-    <mergeCell ref="C2654:G2654"/>
-    <mergeCell ref="C2597:G2597"/>
-    <mergeCell ref="C2598:G2598"/>
-    <mergeCell ref="C2605:G2605"/>
-    <mergeCell ref="C2606:G2606"/>
-    <mergeCell ref="C2612:G2612"/>
-    <mergeCell ref="C2613:G2613"/>
-    <mergeCell ref="C2698:G2698"/>
-    <mergeCell ref="C2699:G2699"/>
-    <mergeCell ref="C2707:G2707"/>
-    <mergeCell ref="C2708:G2708"/>
-    <mergeCell ref="C2717:G2717"/>
-    <mergeCell ref="C2718:G2718"/>
-    <mergeCell ref="C2664:G2664"/>
-    <mergeCell ref="C2665:G2665"/>
-    <mergeCell ref="C2674:G2674"/>
-    <mergeCell ref="C2675:G2675"/>
-    <mergeCell ref="C2691:G2691"/>
-    <mergeCell ref="C2692:G2692"/>
-    <mergeCell ref="C2767:G2767"/>
-    <mergeCell ref="C2768:G2768"/>
-    <mergeCell ref="C2783:G2783"/>
-    <mergeCell ref="C2784:G2784"/>
-    <mergeCell ref="C2794:G2794"/>
-    <mergeCell ref="C2795:G2795"/>
-    <mergeCell ref="C2725:G2725"/>
-    <mergeCell ref="C2726:G2726"/>
-    <mergeCell ref="C2739:G2739"/>
-    <mergeCell ref="C2740:G2740"/>
-    <mergeCell ref="C2750:G2750"/>
-    <mergeCell ref="C2751:G2751"/>
-    <mergeCell ref="C2829:G2829"/>
-    <mergeCell ref="C2830:G2830"/>
-    <mergeCell ref="C2834:G2834"/>
-    <mergeCell ref="C2835:G2835"/>
-    <mergeCell ref="C2844:G2844"/>
-    <mergeCell ref="C2845:G2845"/>
-    <mergeCell ref="C2801:G2801"/>
-    <mergeCell ref="C2802:G2802"/>
-    <mergeCell ref="C2807:G2807"/>
-    <mergeCell ref="C2808:G2808"/>
-    <mergeCell ref="C2815:G2815"/>
-    <mergeCell ref="C2816:G2816"/>
-    <mergeCell ref="C2906:G2906"/>
-    <mergeCell ref="C2907:G2907"/>
-    <mergeCell ref="C2914:G2914"/>
-    <mergeCell ref="C2915:G2915"/>
-    <mergeCell ref="C2933:G2933"/>
-    <mergeCell ref="C2934:G2934"/>
-    <mergeCell ref="C2849:G2849"/>
-    <mergeCell ref="C2850:G2850"/>
-    <mergeCell ref="C2863:G2863"/>
-    <mergeCell ref="C2864:G2864"/>
-    <mergeCell ref="C2874:G2874"/>
-    <mergeCell ref="C2875:G2875"/>
-    <mergeCell ref="C2975:G2975"/>
-    <mergeCell ref="C2976:G2976"/>
-    <mergeCell ref="C2990:G2990"/>
-    <mergeCell ref="C2991:G2991"/>
-    <mergeCell ref="C3000:G3000"/>
-    <mergeCell ref="C3001:G3001"/>
-    <mergeCell ref="C2945:G2945"/>
-    <mergeCell ref="C2946:G2946"/>
-    <mergeCell ref="C2959:G2959"/>
-    <mergeCell ref="C2960:G2960"/>
-    <mergeCell ref="C2968:G2968"/>
-    <mergeCell ref="C2969:G2969"/>
-    <mergeCell ref="C3041:G3041"/>
-    <mergeCell ref="C3042:G3042"/>
-    <mergeCell ref="C3048:G3048"/>
-    <mergeCell ref="C3049:G3049"/>
-    <mergeCell ref="C3055:G3055"/>
-    <mergeCell ref="C3056:G3056"/>
-    <mergeCell ref="C3012:G3012"/>
-    <mergeCell ref="C3013:G3013"/>
-    <mergeCell ref="C3024:G3024"/>
-    <mergeCell ref="C3025:G3025"/>
-    <mergeCell ref="C3036:G3036"/>
-    <mergeCell ref="C3037:G3037"/>
-    <mergeCell ref="C3091:G3091"/>
-    <mergeCell ref="C3092:G3092"/>
-    <mergeCell ref="C3102:G3102"/>
-    <mergeCell ref="C3103:G3103"/>
-    <mergeCell ref="C3117:G3117"/>
-    <mergeCell ref="C3118:G3118"/>
-    <mergeCell ref="C3062:G3062"/>
-    <mergeCell ref="C3063:G3063"/>
-    <mergeCell ref="C3073:G3073"/>
-    <mergeCell ref="C3074:G3074"/>
-    <mergeCell ref="C3081:G3081"/>
-    <mergeCell ref="C3082:G3082"/>
-    <mergeCell ref="C3165:G3165"/>
-    <mergeCell ref="C3166:G3166"/>
-    <mergeCell ref="C3171:G3171"/>
-    <mergeCell ref="C3172:G3172"/>
-    <mergeCell ref="C3178:G3178"/>
-    <mergeCell ref="C3179:G3179"/>
-    <mergeCell ref="C3130:G3130"/>
-    <mergeCell ref="C3131:G3131"/>
-    <mergeCell ref="C3142:G3142"/>
-    <mergeCell ref="C3143:G3143"/>
-    <mergeCell ref="C3157:G3157"/>
-    <mergeCell ref="C3158:G3158"/>
-    <mergeCell ref="C3223:G3223"/>
-    <mergeCell ref="C3224:G3224"/>
-    <mergeCell ref="C3232:G3232"/>
-    <mergeCell ref="C3233:G3233"/>
-    <mergeCell ref="C3241:G3241"/>
-    <mergeCell ref="C3242:G3242"/>
-    <mergeCell ref="C3189:G3189"/>
-    <mergeCell ref="C3190:G3190"/>
-    <mergeCell ref="C3205:G3205"/>
-    <mergeCell ref="C3206:G3206"/>
-    <mergeCell ref="C3215:G3215"/>
-    <mergeCell ref="C3216:G3216"/>
-    <mergeCell ref="C3331:G3331"/>
-    <mergeCell ref="C3332:G3332"/>
-    <mergeCell ref="C3358:G3358"/>
-    <mergeCell ref="C3359:G3359"/>
-    <mergeCell ref="C3367:G3367"/>
-    <mergeCell ref="C3368:G3368"/>
-    <mergeCell ref="C3254:G3254"/>
-    <mergeCell ref="C3255:G3255"/>
-    <mergeCell ref="C3317:G3317"/>
-    <mergeCell ref="C3318:G3318"/>
-    <mergeCell ref="C3324:G3324"/>
-    <mergeCell ref="C3325:G3325"/>
-    <mergeCell ref="C3430:G3430"/>
-    <mergeCell ref="C3431:G3431"/>
-    <mergeCell ref="C3439:G3439"/>
-    <mergeCell ref="C3440:G3440"/>
-    <mergeCell ref="C3444:G3444"/>
-    <mergeCell ref="C3445:G3445"/>
-    <mergeCell ref="C3383:G3383"/>
-    <mergeCell ref="C3384:G3384"/>
-    <mergeCell ref="C3413:G3413"/>
-    <mergeCell ref="C3414:G3414"/>
-    <mergeCell ref="C3421:G3421"/>
-    <mergeCell ref="C3422:G3422"/>
-    <mergeCell ref="C3507:G3507"/>
-    <mergeCell ref="C3508:G3508"/>
-    <mergeCell ref="C3518:G3518"/>
-    <mergeCell ref="C3519:G3519"/>
-    <mergeCell ref="C3540:G3540"/>
-    <mergeCell ref="C3541:G3541"/>
-    <mergeCell ref="C3466:G3466"/>
-    <mergeCell ref="C3467:G3467"/>
-    <mergeCell ref="C3473:G3473"/>
-    <mergeCell ref="C3474:G3474"/>
-    <mergeCell ref="C3487:G3487"/>
-    <mergeCell ref="C3488:G3488"/>
-    <mergeCell ref="C3594:G3594"/>
-    <mergeCell ref="C3595:G3595"/>
-    <mergeCell ref="C3603:G3603"/>
-    <mergeCell ref="C3604:G3604"/>
-    <mergeCell ref="C3611:G3611"/>
-    <mergeCell ref="C3612:G3612"/>
-    <mergeCell ref="C3550:G3550"/>
-    <mergeCell ref="C3551:G3551"/>
-    <mergeCell ref="C3571:G3571"/>
-    <mergeCell ref="C3572:G3572"/>
-    <mergeCell ref="C3581:G3581"/>
-    <mergeCell ref="C3582:G3582"/>
-    <mergeCell ref="C3644:G3644"/>
-    <mergeCell ref="C3652:G3652"/>
-    <mergeCell ref="C3653:G3653"/>
-    <mergeCell ref="C3659:G3659"/>
-    <mergeCell ref="C3660:G3660"/>
-    <mergeCell ref="C3619:G3619"/>
-    <mergeCell ref="C3620:G3620"/>
-    <mergeCell ref="C3630:G3630"/>
-    <mergeCell ref="C3631:G3631"/>
-    <mergeCell ref="C3637:G3637"/>
-    <mergeCell ref="C3638:G3638"/>
     <mergeCell ref="C3763:G3763"/>
     <mergeCell ref="C3764:G3764"/>
     <mergeCell ref="C3776:G3776"/>
@@ -63648,6 +63017,637 @@
     <mergeCell ref="C3691:G3691"/>
     <mergeCell ref="C3692:G3692"/>
     <mergeCell ref="C3643:G3643"/>
+    <mergeCell ref="C3644:G3644"/>
+    <mergeCell ref="C3652:G3652"/>
+    <mergeCell ref="C3653:G3653"/>
+    <mergeCell ref="C3659:G3659"/>
+    <mergeCell ref="C3660:G3660"/>
+    <mergeCell ref="C3619:G3619"/>
+    <mergeCell ref="C3620:G3620"/>
+    <mergeCell ref="C3630:G3630"/>
+    <mergeCell ref="C3631:G3631"/>
+    <mergeCell ref="C3637:G3637"/>
+    <mergeCell ref="C3638:G3638"/>
+    <mergeCell ref="C3594:G3594"/>
+    <mergeCell ref="C3595:G3595"/>
+    <mergeCell ref="C3603:G3603"/>
+    <mergeCell ref="C3604:G3604"/>
+    <mergeCell ref="C3611:G3611"/>
+    <mergeCell ref="C3612:G3612"/>
+    <mergeCell ref="C3550:G3550"/>
+    <mergeCell ref="C3551:G3551"/>
+    <mergeCell ref="C3571:G3571"/>
+    <mergeCell ref="C3572:G3572"/>
+    <mergeCell ref="C3581:G3581"/>
+    <mergeCell ref="C3582:G3582"/>
+    <mergeCell ref="C3507:G3507"/>
+    <mergeCell ref="C3508:G3508"/>
+    <mergeCell ref="C3518:G3518"/>
+    <mergeCell ref="C3519:G3519"/>
+    <mergeCell ref="C3540:G3540"/>
+    <mergeCell ref="C3541:G3541"/>
+    <mergeCell ref="C3466:G3466"/>
+    <mergeCell ref="C3467:G3467"/>
+    <mergeCell ref="C3473:G3473"/>
+    <mergeCell ref="C3474:G3474"/>
+    <mergeCell ref="C3487:G3487"/>
+    <mergeCell ref="C3488:G3488"/>
+    <mergeCell ref="C3430:G3430"/>
+    <mergeCell ref="C3431:G3431"/>
+    <mergeCell ref="C3439:G3439"/>
+    <mergeCell ref="C3440:G3440"/>
+    <mergeCell ref="C3444:G3444"/>
+    <mergeCell ref="C3445:G3445"/>
+    <mergeCell ref="C3383:G3383"/>
+    <mergeCell ref="C3384:G3384"/>
+    <mergeCell ref="C3413:G3413"/>
+    <mergeCell ref="C3414:G3414"/>
+    <mergeCell ref="C3421:G3421"/>
+    <mergeCell ref="C3422:G3422"/>
+    <mergeCell ref="C3331:G3331"/>
+    <mergeCell ref="C3332:G3332"/>
+    <mergeCell ref="C3358:G3358"/>
+    <mergeCell ref="C3359:G3359"/>
+    <mergeCell ref="C3367:G3367"/>
+    <mergeCell ref="C3368:G3368"/>
+    <mergeCell ref="C3254:G3254"/>
+    <mergeCell ref="C3255:G3255"/>
+    <mergeCell ref="C3317:G3317"/>
+    <mergeCell ref="C3318:G3318"/>
+    <mergeCell ref="C3324:G3324"/>
+    <mergeCell ref="C3325:G3325"/>
+    <mergeCell ref="C3223:G3223"/>
+    <mergeCell ref="C3224:G3224"/>
+    <mergeCell ref="C3232:G3232"/>
+    <mergeCell ref="C3233:G3233"/>
+    <mergeCell ref="C3241:G3241"/>
+    <mergeCell ref="C3242:G3242"/>
+    <mergeCell ref="C3189:G3189"/>
+    <mergeCell ref="C3190:G3190"/>
+    <mergeCell ref="C3205:G3205"/>
+    <mergeCell ref="C3206:G3206"/>
+    <mergeCell ref="C3215:G3215"/>
+    <mergeCell ref="C3216:G3216"/>
+    <mergeCell ref="C3165:G3165"/>
+    <mergeCell ref="C3166:G3166"/>
+    <mergeCell ref="C3171:G3171"/>
+    <mergeCell ref="C3172:G3172"/>
+    <mergeCell ref="C3178:G3178"/>
+    <mergeCell ref="C3179:G3179"/>
+    <mergeCell ref="C3130:G3130"/>
+    <mergeCell ref="C3131:G3131"/>
+    <mergeCell ref="C3142:G3142"/>
+    <mergeCell ref="C3143:G3143"/>
+    <mergeCell ref="C3157:G3157"/>
+    <mergeCell ref="C3158:G3158"/>
+    <mergeCell ref="C3091:G3091"/>
+    <mergeCell ref="C3092:G3092"/>
+    <mergeCell ref="C3102:G3102"/>
+    <mergeCell ref="C3103:G3103"/>
+    <mergeCell ref="C3117:G3117"/>
+    <mergeCell ref="C3118:G3118"/>
+    <mergeCell ref="C3062:G3062"/>
+    <mergeCell ref="C3063:G3063"/>
+    <mergeCell ref="C3073:G3073"/>
+    <mergeCell ref="C3074:G3074"/>
+    <mergeCell ref="C3081:G3081"/>
+    <mergeCell ref="C3082:G3082"/>
+    <mergeCell ref="C3041:G3041"/>
+    <mergeCell ref="C3042:G3042"/>
+    <mergeCell ref="C3048:G3048"/>
+    <mergeCell ref="C3049:G3049"/>
+    <mergeCell ref="C3055:G3055"/>
+    <mergeCell ref="C3056:G3056"/>
+    <mergeCell ref="C3012:G3012"/>
+    <mergeCell ref="C3013:G3013"/>
+    <mergeCell ref="C3024:G3024"/>
+    <mergeCell ref="C3025:G3025"/>
+    <mergeCell ref="C3036:G3036"/>
+    <mergeCell ref="C3037:G3037"/>
+    <mergeCell ref="C2975:G2975"/>
+    <mergeCell ref="C2976:G2976"/>
+    <mergeCell ref="C2990:G2990"/>
+    <mergeCell ref="C2991:G2991"/>
+    <mergeCell ref="C3000:G3000"/>
+    <mergeCell ref="C3001:G3001"/>
+    <mergeCell ref="C2945:G2945"/>
+    <mergeCell ref="C2946:G2946"/>
+    <mergeCell ref="C2959:G2959"/>
+    <mergeCell ref="C2960:G2960"/>
+    <mergeCell ref="C2968:G2968"/>
+    <mergeCell ref="C2969:G2969"/>
+    <mergeCell ref="C2906:G2906"/>
+    <mergeCell ref="C2907:G2907"/>
+    <mergeCell ref="C2914:G2914"/>
+    <mergeCell ref="C2915:G2915"/>
+    <mergeCell ref="C2933:G2933"/>
+    <mergeCell ref="C2934:G2934"/>
+    <mergeCell ref="C2849:G2849"/>
+    <mergeCell ref="C2850:G2850"/>
+    <mergeCell ref="C2863:G2863"/>
+    <mergeCell ref="C2864:G2864"/>
+    <mergeCell ref="C2874:G2874"/>
+    <mergeCell ref="C2875:G2875"/>
+    <mergeCell ref="C2829:G2829"/>
+    <mergeCell ref="C2830:G2830"/>
+    <mergeCell ref="C2834:G2834"/>
+    <mergeCell ref="C2835:G2835"/>
+    <mergeCell ref="C2844:G2844"/>
+    <mergeCell ref="C2845:G2845"/>
+    <mergeCell ref="C2801:G2801"/>
+    <mergeCell ref="C2802:G2802"/>
+    <mergeCell ref="C2807:G2807"/>
+    <mergeCell ref="C2808:G2808"/>
+    <mergeCell ref="C2815:G2815"/>
+    <mergeCell ref="C2816:G2816"/>
+    <mergeCell ref="C2767:G2767"/>
+    <mergeCell ref="C2768:G2768"/>
+    <mergeCell ref="C2783:G2783"/>
+    <mergeCell ref="C2784:G2784"/>
+    <mergeCell ref="C2794:G2794"/>
+    <mergeCell ref="C2795:G2795"/>
+    <mergeCell ref="C2725:G2725"/>
+    <mergeCell ref="C2726:G2726"/>
+    <mergeCell ref="C2739:G2739"/>
+    <mergeCell ref="C2740:G2740"/>
+    <mergeCell ref="C2750:G2750"/>
+    <mergeCell ref="C2751:G2751"/>
+    <mergeCell ref="C2698:G2698"/>
+    <mergeCell ref="C2699:G2699"/>
+    <mergeCell ref="C2707:G2707"/>
+    <mergeCell ref="C2708:G2708"/>
+    <mergeCell ref="C2717:G2717"/>
+    <mergeCell ref="C2718:G2718"/>
+    <mergeCell ref="C2664:G2664"/>
+    <mergeCell ref="C2665:G2665"/>
+    <mergeCell ref="C2674:G2674"/>
+    <mergeCell ref="C2675:G2675"/>
+    <mergeCell ref="C2691:G2691"/>
+    <mergeCell ref="C2692:G2692"/>
+    <mergeCell ref="C2637:G2637"/>
+    <mergeCell ref="C2638:G2638"/>
+    <mergeCell ref="C2645:G2645"/>
+    <mergeCell ref="C2646:G2646"/>
+    <mergeCell ref="C2653:G2653"/>
+    <mergeCell ref="C2654:G2654"/>
+    <mergeCell ref="C2597:G2597"/>
+    <mergeCell ref="C2598:G2598"/>
+    <mergeCell ref="C2605:G2605"/>
+    <mergeCell ref="C2606:G2606"/>
+    <mergeCell ref="C2612:G2612"/>
+    <mergeCell ref="C2613:G2613"/>
+    <mergeCell ref="C2559:G2559"/>
+    <mergeCell ref="C2560:G2560"/>
+    <mergeCell ref="C2569:G2569"/>
+    <mergeCell ref="C2570:G2570"/>
+    <mergeCell ref="C2584:G2584"/>
+    <mergeCell ref="C2585:G2585"/>
+    <mergeCell ref="C2530:G2530"/>
+    <mergeCell ref="C2531:G2531"/>
+    <mergeCell ref="C2539:G2539"/>
+    <mergeCell ref="C2540:G2540"/>
+    <mergeCell ref="C2547:G2547"/>
+    <mergeCell ref="C2548:G2548"/>
+    <mergeCell ref="C2492:G2492"/>
+    <mergeCell ref="C2493:G2493"/>
+    <mergeCell ref="C2506:G2506"/>
+    <mergeCell ref="C2507:G2507"/>
+    <mergeCell ref="C2519:G2519"/>
+    <mergeCell ref="C2520:G2520"/>
+    <mergeCell ref="C2462:G2462"/>
+    <mergeCell ref="C2463:G2463"/>
+    <mergeCell ref="C2469:G2469"/>
+    <mergeCell ref="C2470:G2470"/>
+    <mergeCell ref="C2482:G2482"/>
+    <mergeCell ref="C2483:G2483"/>
+    <mergeCell ref="C2433:G2433"/>
+    <mergeCell ref="C2434:G2434"/>
+    <mergeCell ref="C2440:G2440"/>
+    <mergeCell ref="C2441:G2441"/>
+    <mergeCell ref="C2454:G2454"/>
+    <mergeCell ref="C2455:G2455"/>
+    <mergeCell ref="C2409:G2409"/>
+    <mergeCell ref="C2410:G2410"/>
+    <mergeCell ref="C2417:G2417"/>
+    <mergeCell ref="C2418:G2418"/>
+    <mergeCell ref="C2425:G2425"/>
+    <mergeCell ref="C2426:G2426"/>
+    <mergeCell ref="C2383:G2383"/>
+    <mergeCell ref="C2384:G2384"/>
+    <mergeCell ref="C2391:G2391"/>
+    <mergeCell ref="C2392:G2392"/>
+    <mergeCell ref="C2399:G2399"/>
+    <mergeCell ref="C2400:G2400"/>
+    <mergeCell ref="C2358:G2358"/>
+    <mergeCell ref="C2359:G2359"/>
+    <mergeCell ref="C2366:G2366"/>
+    <mergeCell ref="C2367:G2367"/>
+    <mergeCell ref="C2377:G2377"/>
+    <mergeCell ref="C2378:G2378"/>
+    <mergeCell ref="C2289:G2289"/>
+    <mergeCell ref="C2290:G2290"/>
+    <mergeCell ref="C2337:G2337"/>
+    <mergeCell ref="C2338:G2338"/>
+    <mergeCell ref="C2351:G2351"/>
+    <mergeCell ref="C2352:G2352"/>
+    <mergeCell ref="C2257:G2257"/>
+    <mergeCell ref="C2258:G2258"/>
+    <mergeCell ref="C2274:G2274"/>
+    <mergeCell ref="C2275:G2275"/>
+    <mergeCell ref="C2281:G2281"/>
+    <mergeCell ref="C2282:G2282"/>
+    <mergeCell ref="C2228:G2228"/>
+    <mergeCell ref="C2229:G2229"/>
+    <mergeCell ref="C2242:G2242"/>
+    <mergeCell ref="C2243:G2243"/>
+    <mergeCell ref="C2250:G2250"/>
+    <mergeCell ref="C2251:G2251"/>
+    <mergeCell ref="C2194:G2194"/>
+    <mergeCell ref="C2195:G2195"/>
+    <mergeCell ref="C2210:G2210"/>
+    <mergeCell ref="C2211:G2211"/>
+    <mergeCell ref="C2218:G2218"/>
+    <mergeCell ref="C2219:G2219"/>
+    <mergeCell ref="C2173:G2173"/>
+    <mergeCell ref="C2174:G2174"/>
+    <mergeCell ref="C2179:G2179"/>
+    <mergeCell ref="C2180:G2180"/>
+    <mergeCell ref="C2186:G2186"/>
+    <mergeCell ref="C2187:G2187"/>
+    <mergeCell ref="C2123:G2123"/>
+    <mergeCell ref="C2124:G2124"/>
+    <mergeCell ref="C2131:G2131"/>
+    <mergeCell ref="C2132:G2132"/>
+    <mergeCell ref="C2138:G2138"/>
+    <mergeCell ref="C2139:G2139"/>
+    <mergeCell ref="C2091:G2091"/>
+    <mergeCell ref="C2092:G2092"/>
+    <mergeCell ref="C2103:G2103"/>
+    <mergeCell ref="C2104:G2104"/>
+    <mergeCell ref="C2114:G2114"/>
+    <mergeCell ref="C2115:G2115"/>
+    <mergeCell ref="C2031:G2031"/>
+    <mergeCell ref="C2032:G2032"/>
+    <mergeCell ref="C2041:G2041"/>
+    <mergeCell ref="C2042:G2042"/>
+    <mergeCell ref="C2079:G2079"/>
+    <mergeCell ref="C2080:G2080"/>
+    <mergeCell ref="C1993:G1993"/>
+    <mergeCell ref="C1994:G1994"/>
+    <mergeCell ref="C2001:G2001"/>
+    <mergeCell ref="C2002:G2002"/>
+    <mergeCell ref="C2023:G2023"/>
+    <mergeCell ref="C2024:G2024"/>
+    <mergeCell ref="C1952:G1952"/>
+    <mergeCell ref="C1953:G1953"/>
+    <mergeCell ref="C1964:G1964"/>
+    <mergeCell ref="C1965:G1965"/>
+    <mergeCell ref="C1984:G1984"/>
+    <mergeCell ref="C1985:G1985"/>
+    <mergeCell ref="C1918:G1918"/>
+    <mergeCell ref="C1919:G1919"/>
+    <mergeCell ref="C1924:G1924"/>
+    <mergeCell ref="C1925:G1925"/>
+    <mergeCell ref="C1942:G1942"/>
+    <mergeCell ref="C1943:G1943"/>
+    <mergeCell ref="C1883:G1883"/>
+    <mergeCell ref="C1884:G1884"/>
+    <mergeCell ref="C1893:G1893"/>
+    <mergeCell ref="C1894:G1894"/>
+    <mergeCell ref="C1912:G1912"/>
+    <mergeCell ref="C1913:G1913"/>
+    <mergeCell ref="C1856:G1856"/>
+    <mergeCell ref="C1857:G1857"/>
+    <mergeCell ref="C1865:G1865"/>
+    <mergeCell ref="C1866:G1866"/>
+    <mergeCell ref="C1872:G1872"/>
+    <mergeCell ref="C1873:G1873"/>
+    <mergeCell ref="C1821:G1821"/>
+    <mergeCell ref="C1822:G1822"/>
+    <mergeCell ref="C1830:G1830"/>
+    <mergeCell ref="C1831:G1831"/>
+    <mergeCell ref="C1840:G1840"/>
+    <mergeCell ref="C1777:G1777"/>
+    <mergeCell ref="C1778:G1778"/>
+    <mergeCell ref="C1789:G1789"/>
+    <mergeCell ref="C1790:G1790"/>
+    <mergeCell ref="C1804:G1804"/>
+    <mergeCell ref="C1805:G1805"/>
+    <mergeCell ref="C1734:G1734"/>
+    <mergeCell ref="C1735:G1735"/>
+    <mergeCell ref="C1745:G1745"/>
+    <mergeCell ref="C1746:G1746"/>
+    <mergeCell ref="C1763:G1763"/>
+    <mergeCell ref="C1764:G1764"/>
+    <mergeCell ref="C1703:G1703"/>
+    <mergeCell ref="C1704:G1704"/>
+    <mergeCell ref="C1713:G1713"/>
+    <mergeCell ref="C1714:G1714"/>
+    <mergeCell ref="C1723:G1723"/>
+    <mergeCell ref="C1724:G1724"/>
+    <mergeCell ref="C1670:G1670"/>
+    <mergeCell ref="C1671:G1671"/>
+    <mergeCell ref="C1679:G1679"/>
+    <mergeCell ref="C1680:G1680"/>
+    <mergeCell ref="C1688:G1688"/>
+    <mergeCell ref="C1689:G1689"/>
+    <mergeCell ref="C1639:G1639"/>
+    <mergeCell ref="C1640:G1640"/>
+    <mergeCell ref="C1645:G1645"/>
+    <mergeCell ref="C1646:G1646"/>
+    <mergeCell ref="C1651:G1651"/>
+    <mergeCell ref="C1652:G1652"/>
+    <mergeCell ref="C1600:G1600"/>
+    <mergeCell ref="C1601:G1601"/>
+    <mergeCell ref="C1614:G1614"/>
+    <mergeCell ref="C1615:G1615"/>
+    <mergeCell ref="C1626:G1626"/>
+    <mergeCell ref="C1627:G1627"/>
+    <mergeCell ref="C1553:G1553"/>
+    <mergeCell ref="C1554:G1554"/>
+    <mergeCell ref="C1572:G1572"/>
+    <mergeCell ref="C1573:G1573"/>
+    <mergeCell ref="C1591:G1591"/>
+    <mergeCell ref="C1592:G1592"/>
+    <mergeCell ref="C1516:G1516"/>
+    <mergeCell ref="C1517:G1517"/>
+    <mergeCell ref="C1523:G1523"/>
+    <mergeCell ref="C1524:G1524"/>
+    <mergeCell ref="C1540:G1540"/>
+    <mergeCell ref="C1541:G1541"/>
+    <mergeCell ref="C1491:G1491"/>
+    <mergeCell ref="C1492:G1492"/>
+    <mergeCell ref="C1497:G1497"/>
+    <mergeCell ref="C1498:G1498"/>
+    <mergeCell ref="C1508:G1508"/>
+    <mergeCell ref="C1509:G1509"/>
+    <mergeCell ref="C1466:G1466"/>
+    <mergeCell ref="C1467:G1467"/>
+    <mergeCell ref="C1475:G1475"/>
+    <mergeCell ref="C1476:G1476"/>
+    <mergeCell ref="C1482:G1482"/>
+    <mergeCell ref="C1483:G1483"/>
+    <mergeCell ref="C1433:G1433"/>
+    <mergeCell ref="C1434:G1434"/>
+    <mergeCell ref="C1442:G1442"/>
+    <mergeCell ref="C1443:G1443"/>
+    <mergeCell ref="C1459:G1459"/>
+    <mergeCell ref="C1460:G1460"/>
+    <mergeCell ref="C1398:G1398"/>
+    <mergeCell ref="C1399:G1399"/>
+    <mergeCell ref="C1406:G1406"/>
+    <mergeCell ref="C1407:G1407"/>
+    <mergeCell ref="C1417:G1417"/>
+    <mergeCell ref="C1418:G1418"/>
+    <mergeCell ref="C1368:G1368"/>
+    <mergeCell ref="C1369:G1369"/>
+    <mergeCell ref="C1381:G1381"/>
+    <mergeCell ref="C1382:G1382"/>
+    <mergeCell ref="C1390:G1390"/>
+    <mergeCell ref="C1391:G1391"/>
+    <mergeCell ref="C1336:G1336"/>
+    <mergeCell ref="C1337:G1337"/>
+    <mergeCell ref="C1345:G1345"/>
+    <mergeCell ref="C1346:G1346"/>
+    <mergeCell ref="C1361:G1361"/>
+    <mergeCell ref="C1362:G1362"/>
+    <mergeCell ref="C1319:G1319"/>
+    <mergeCell ref="C1320:G1320"/>
+    <mergeCell ref="C1324:G1324"/>
+    <mergeCell ref="C1325:G1325"/>
+    <mergeCell ref="C1330:G1330"/>
+    <mergeCell ref="C1331:G1331"/>
+    <mergeCell ref="C1281:G1281"/>
+    <mergeCell ref="C1282:G1282"/>
+    <mergeCell ref="C1297:G1297"/>
+    <mergeCell ref="C1298:G1298"/>
+    <mergeCell ref="C1309:G1309"/>
+    <mergeCell ref="C1310:G1310"/>
+    <mergeCell ref="C1258:G1258"/>
+    <mergeCell ref="C1259:G1259"/>
+    <mergeCell ref="C1267:G1267"/>
+    <mergeCell ref="C1268:G1268"/>
+    <mergeCell ref="C1274:G1274"/>
+    <mergeCell ref="C1275:G1275"/>
+    <mergeCell ref="C1228:G1228"/>
+    <mergeCell ref="C1229:G1229"/>
+    <mergeCell ref="C1239:G1239"/>
+    <mergeCell ref="C1240:G1240"/>
+    <mergeCell ref="C1250:G1250"/>
+    <mergeCell ref="C1251:G1251"/>
+    <mergeCell ref="C1186:G1186"/>
+    <mergeCell ref="C1187:G1187"/>
+    <mergeCell ref="C1199:G1199"/>
+    <mergeCell ref="C1200:G1200"/>
+    <mergeCell ref="C1221:G1221"/>
+    <mergeCell ref="C1222:G1222"/>
+    <mergeCell ref="C1150:G1150"/>
+    <mergeCell ref="C1151:G1151"/>
+    <mergeCell ref="C1163:G1163"/>
+    <mergeCell ref="C1164:G1164"/>
+    <mergeCell ref="C1178:G1178"/>
+    <mergeCell ref="C1179:G1179"/>
+    <mergeCell ref="C1116:G1116"/>
+    <mergeCell ref="C1117:G1117"/>
+    <mergeCell ref="C1127:G1127"/>
+    <mergeCell ref="C1128:G1128"/>
+    <mergeCell ref="C1142:G1142"/>
+    <mergeCell ref="C1143:G1143"/>
+    <mergeCell ref="C1087:G1087"/>
+    <mergeCell ref="C1088:G1088"/>
+    <mergeCell ref="C1099:G1099"/>
+    <mergeCell ref="C1100:G1100"/>
+    <mergeCell ref="C1106:G1106"/>
+    <mergeCell ref="C1107:G1107"/>
+    <mergeCell ref="C1013:G1013"/>
+    <mergeCell ref="C1014:G1014"/>
+    <mergeCell ref="C1021:G1021"/>
+    <mergeCell ref="C1022:G1022"/>
+    <mergeCell ref="C1069:G1069"/>
+    <mergeCell ref="C1070:G1070"/>
+    <mergeCell ref="C987:G987"/>
+    <mergeCell ref="C988:G988"/>
+    <mergeCell ref="C997:G997"/>
+    <mergeCell ref="C998:G998"/>
+    <mergeCell ref="C1003:G1003"/>
+    <mergeCell ref="C1004:G1004"/>
+    <mergeCell ref="C955:G955"/>
+    <mergeCell ref="C956:G956"/>
+    <mergeCell ref="C965:G965"/>
+    <mergeCell ref="C966:G966"/>
+    <mergeCell ref="C975:G975"/>
+    <mergeCell ref="C976:G976"/>
+    <mergeCell ref="C930:G930"/>
+    <mergeCell ref="C931:G931"/>
+    <mergeCell ref="C936:G936"/>
+    <mergeCell ref="C937:G937"/>
+    <mergeCell ref="C944:G944"/>
+    <mergeCell ref="C945:G945"/>
+    <mergeCell ref="C898:G898"/>
+    <mergeCell ref="C899:G899"/>
+    <mergeCell ref="C907:G907"/>
+    <mergeCell ref="C908:G908"/>
+    <mergeCell ref="C919:G919"/>
+    <mergeCell ref="C920:G920"/>
+    <mergeCell ref="C876:G876"/>
+    <mergeCell ref="C877:G877"/>
+    <mergeCell ref="C884:G884"/>
+    <mergeCell ref="C885:G885"/>
+    <mergeCell ref="C892:G892"/>
+    <mergeCell ref="C893:G893"/>
+    <mergeCell ref="C848:G848"/>
+    <mergeCell ref="C849:G849"/>
+    <mergeCell ref="C858:G858"/>
+    <mergeCell ref="C859:G859"/>
+    <mergeCell ref="C868:G868"/>
+    <mergeCell ref="C869:G869"/>
+    <mergeCell ref="C817:G817"/>
+    <mergeCell ref="C818:G818"/>
+    <mergeCell ref="C827:G827"/>
+    <mergeCell ref="C828:G828"/>
+    <mergeCell ref="C837:G837"/>
+    <mergeCell ref="C838:G838"/>
+    <mergeCell ref="C792:G792"/>
+    <mergeCell ref="C793:G793"/>
+    <mergeCell ref="C802:G802"/>
+    <mergeCell ref="C803:G803"/>
+    <mergeCell ref="C808:G808"/>
+    <mergeCell ref="C809:G809"/>
+    <mergeCell ref="C752:G752"/>
+    <mergeCell ref="C753:G753"/>
+    <mergeCell ref="C766:G766"/>
+    <mergeCell ref="C767:G767"/>
+    <mergeCell ref="C774:G774"/>
+    <mergeCell ref="C775:G775"/>
+    <mergeCell ref="C733:G733"/>
+    <mergeCell ref="C734:G734"/>
+    <mergeCell ref="C742:G742"/>
+    <mergeCell ref="C743:G743"/>
+    <mergeCell ref="C702:G702"/>
+    <mergeCell ref="C703:G703"/>
+    <mergeCell ref="C710:G710"/>
+    <mergeCell ref="C711:G711"/>
+    <mergeCell ref="C721:G721"/>
+    <mergeCell ref="C722:G722"/>
+    <mergeCell ref="C661:G661"/>
+    <mergeCell ref="C662:G662"/>
+    <mergeCell ref="C683:G683"/>
+    <mergeCell ref="C684:G684"/>
+    <mergeCell ref="C692:G692"/>
+    <mergeCell ref="C693:G693"/>
+    <mergeCell ref="C625:G625"/>
+    <mergeCell ref="C626:G626"/>
+    <mergeCell ref="C637:G637"/>
+    <mergeCell ref="C638:G638"/>
+    <mergeCell ref="C644:G644"/>
+    <mergeCell ref="C645:G645"/>
+    <mergeCell ref="C598:G598"/>
+    <mergeCell ref="C599:G599"/>
+    <mergeCell ref="C607:G607"/>
+    <mergeCell ref="C608:G608"/>
+    <mergeCell ref="C615:G615"/>
+    <mergeCell ref="C616:G616"/>
+    <mergeCell ref="C575:G575"/>
+    <mergeCell ref="C576:G576"/>
+    <mergeCell ref="C583:G583"/>
+    <mergeCell ref="C584:G584"/>
+    <mergeCell ref="C590:G590"/>
+    <mergeCell ref="C591:G591"/>
+    <mergeCell ref="C527:G527"/>
+    <mergeCell ref="C528:G528"/>
+    <mergeCell ref="C543:G543"/>
+    <mergeCell ref="C544:G544"/>
+    <mergeCell ref="C567:G567"/>
+    <mergeCell ref="C568:G568"/>
+    <mergeCell ref="C505:G505"/>
+    <mergeCell ref="C506:G506"/>
+    <mergeCell ref="C512:G512"/>
+    <mergeCell ref="C519:G519"/>
+    <mergeCell ref="C520:G520"/>
+    <mergeCell ref="C465:G465"/>
+    <mergeCell ref="C466:G466"/>
+    <mergeCell ref="C474:G474"/>
+    <mergeCell ref="C475:G475"/>
+    <mergeCell ref="C495:G495"/>
+    <mergeCell ref="C496:G496"/>
+    <mergeCell ref="C444:G444"/>
+    <mergeCell ref="C445:G445"/>
+    <mergeCell ref="C452:G452"/>
+    <mergeCell ref="C453:G453"/>
+    <mergeCell ref="C459:G459"/>
+    <mergeCell ref="C460:G460"/>
+    <mergeCell ref="C421:G421"/>
+    <mergeCell ref="C422:G422"/>
+    <mergeCell ref="C427:G427"/>
+    <mergeCell ref="C428:G428"/>
+    <mergeCell ref="C434:G434"/>
+    <mergeCell ref="C435:G435"/>
+    <mergeCell ref="C378:G378"/>
+    <mergeCell ref="C379:G379"/>
+    <mergeCell ref="C385:G385"/>
+    <mergeCell ref="C386:G386"/>
+    <mergeCell ref="C403:G403"/>
+    <mergeCell ref="C404:G404"/>
+    <mergeCell ref="C326:G326"/>
+    <mergeCell ref="C327:G327"/>
+    <mergeCell ref="C356:G356"/>
+    <mergeCell ref="C357:G357"/>
+    <mergeCell ref="C369:G369"/>
+    <mergeCell ref="C370:G370"/>
+    <mergeCell ref="C302:G302"/>
+    <mergeCell ref="C303:G303"/>
+    <mergeCell ref="C310:G310"/>
+    <mergeCell ref="C311:G311"/>
+    <mergeCell ref="C319:G319"/>
+    <mergeCell ref="C320:G320"/>
+    <mergeCell ref="C275:G275"/>
+    <mergeCell ref="C276:G276"/>
+    <mergeCell ref="C284:G284"/>
+    <mergeCell ref="C285:G285"/>
+    <mergeCell ref="C294:G294"/>
+    <mergeCell ref="C295:G295"/>
+    <mergeCell ref="C248:G248"/>
+    <mergeCell ref="C249:G249"/>
+    <mergeCell ref="C255:G255"/>
+    <mergeCell ref="C256:G256"/>
+    <mergeCell ref="C264:G264"/>
+    <mergeCell ref="C265:G265"/>
+    <mergeCell ref="C200:G200"/>
+    <mergeCell ref="C201:G201"/>
+    <mergeCell ref="C217:G217"/>
+    <mergeCell ref="C218:G218"/>
+    <mergeCell ref="C232:G232"/>
+    <mergeCell ref="C233:G233"/>
+    <mergeCell ref="C175:G175"/>
+    <mergeCell ref="C176:G176"/>
+    <mergeCell ref="C183:G183"/>
+    <mergeCell ref="C184:G184"/>
+    <mergeCell ref="C190:G190"/>
+    <mergeCell ref="C191:G191"/>
+    <mergeCell ref="C147:G147"/>
+    <mergeCell ref="C148:G148"/>
+    <mergeCell ref="C154:G154"/>
+    <mergeCell ref="C155:G155"/>
+    <mergeCell ref="C162:G162"/>
+    <mergeCell ref="C163:G163"/>
+    <mergeCell ref="C91:G91"/>
+    <mergeCell ref="C92:G92"/>
+    <mergeCell ref="C130:G130"/>
+    <mergeCell ref="C131:G131"/>
+    <mergeCell ref="C138:G138"/>
+    <mergeCell ref="C139:G139"/>
+    <mergeCell ref="C55:G55"/>
+    <mergeCell ref="C56:G56"/>
+    <mergeCell ref="C69:G69"/>
+    <mergeCell ref="C70:G70"/>
+    <mergeCell ref="C83:G83"/>
+    <mergeCell ref="C84:G84"/>
+    <mergeCell ref="C7:G7"/>
+    <mergeCell ref="C8:G8"/>
+    <mergeCell ref="C31:G31"/>
+    <mergeCell ref="C32:G32"/>
+    <mergeCell ref="C42:G42"/>
+    <mergeCell ref="C43:G43"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>